<commit_message>
updated graph Figure 5
</commit_message>
<xml_diff>
--- a/Supporting Information 2_PlasticFADE.xlsx
+++ b/Supporting Information 2_PlasticFADE.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nadsad/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nadsad/Documents/GitHub/PlasticFADE/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{51392C1F-3171-A743-BBD9-7FA4DBB86A80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FE15425-E3AC-C747-9E0F-A512F03DF2BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17020" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29420" yWindow="-380" windowWidth="38400" windowHeight="21000" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover sheet" sheetId="14" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3480" uniqueCount="1017">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3549" uniqueCount="1058">
   <si>
     <t>Model interface</t>
   </si>
@@ -6398,6 +6398,129 @@
   </si>
   <si>
     <t>Yibo Tang, Nadim Saadi, Jérôme Lavoie, Anne-Marie Boulay</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>SA:V=</t>
+  </si>
+  <si>
+    <t>95_min</t>
+  </si>
+  <si>
+    <t>95_max</t>
+  </si>
+  <si>
+    <t>Highest higher limit of 95CI values (for the dots on the right)</t>
+  </si>
+  <si>
+    <t>Lowest lower limit of 95CI values (for the dots on the right)</t>
+  </si>
+  <si>
+    <t>k_all_pp_1</t>
+  </si>
+  <si>
+    <t>k_all_pp_10</t>
+  </si>
+  <si>
+    <t>k_all_pp_100</t>
+  </si>
+  <si>
+    <t>k_all_pp_1000</t>
+  </si>
+  <si>
+    <t>k_all_pp_5000</t>
+  </si>
+  <si>
+    <t>k_all_ps_1</t>
+  </si>
+  <si>
+    <t>k_all_ps_10</t>
+  </si>
+  <si>
+    <t>k_all_ps_100</t>
+  </si>
+  <si>
+    <t>k_all_ps_1000</t>
+  </si>
+  <si>
+    <t>k_all_ps_5000</t>
+  </si>
+  <si>
+    <t>k_all_eps_1</t>
+  </si>
+  <si>
+    <t>k_all_eps_10</t>
+  </si>
+  <si>
+    <t>k_all_eps_100</t>
+  </si>
+  <si>
+    <t>k_all_eps_1000</t>
+  </si>
+  <si>
+    <t>k_all_eps_5000</t>
+  </si>
+  <si>
+    <t>k_all_hdpe_1</t>
+  </si>
+  <si>
+    <t>k_all_hdpe_5000</t>
+  </si>
+  <si>
+    <t>k_all_hdpe_1000</t>
+  </si>
+  <si>
+    <t>k_all_hdpe_100</t>
+  </si>
+  <si>
+    <t>k_all_hdpe_10</t>
+  </si>
+  <si>
+    <t>k_all_ldpe_1</t>
+  </si>
+  <si>
+    <t>k_all_ldpe_10</t>
+  </si>
+  <si>
+    <t>k_all_ldpe_100</t>
+  </si>
+  <si>
+    <t>k_all_ldpe_1000</t>
+  </si>
+  <si>
+    <t>k_all_ldpe_5000</t>
+  </si>
+  <si>
+    <t>k_all_pe_1</t>
+  </si>
+  <si>
+    <t>k_all_pe_10</t>
+  </si>
+  <si>
+    <t>k_all_pe_100</t>
+  </si>
+  <si>
+    <t>k_all_pe_1000</t>
+  </si>
+  <si>
+    <t>k_all_pe_5000</t>
+  </si>
+  <si>
+    <t>k_all_pet_1</t>
+  </si>
+  <si>
+    <t>k_all_pet_10</t>
+  </si>
+  <si>
+    <t>k_all_pet_100</t>
+  </si>
+  <si>
+    <t>k_all_pet_1000</t>
+  </si>
+  <si>
+    <t>k_all_pet_5000</t>
   </si>
 </sst>
 </file>
@@ -6660,7 +6783,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -6715,11 +6838,108 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -6729,7 +6949,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="223">
+  <cellXfs count="257">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -7305,10 +7525,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -7318,9 +7541,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -7365,6 +7585,9 @@
     <xf numFmtId="11" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -7380,21 +7603,191 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="11" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="1" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
@@ -9811,7 +10204,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF8DA02B-07F9-AF4D-BDCD-88DA687C4C21}">
-  <dimension ref="A1:V25"/>
+  <dimension ref="A1:BG50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="15.83203125" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.83203125" style="4" customWidth="1"/>
@@ -9824,17 +10217,166 @@
     <col min="12" max="12" width="20.83203125" style="4" customWidth="1"/>
     <col min="13" max="13" width="18.83203125" style="4" customWidth="1"/>
     <col min="14" max="21" width="15.83203125" style="4"/>
-    <col min="22" max="22" width="22.33203125" style="4" customWidth="1"/>
-    <col min="23" max="16384" width="15.83203125" style="4"/>
+    <col min="22" max="24" width="22.33203125" style="4" customWidth="1"/>
+    <col min="25" max="16384" width="15.83203125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="158" t="s">
         <v>1003</v>
       </c>
       <c r="B1" s="158"/>
-    </row>
-    <row r="2" spans="1:22" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V1" s="4" t="s">
+        <v>1018</v>
+      </c>
+      <c r="W1" s="225" t="s">
+        <v>1022</v>
+      </c>
+      <c r="X1" s="227" t="s">
+        <v>1021</v>
+      </c>
+      <c r="Y1" s="225">
+        <f>3/(1/2/10000)</f>
+        <v>60000</v>
+      </c>
+      <c r="Z1" s="226">
+        <f>3/(10/2/10000)</f>
+        <v>6000</v>
+      </c>
+      <c r="AA1" s="226">
+        <f>3/(100/2/10000)</f>
+        <v>600</v>
+      </c>
+      <c r="AB1" s="226">
+        <f>3/(1000/2/10000)</f>
+        <v>60</v>
+      </c>
+      <c r="AC1" s="227">
+        <f>3/(5000/2/10000)</f>
+        <v>12</v>
+      </c>
+      <c r="AD1" s="225">
+        <f>3/(1/2/10000)</f>
+        <v>60000</v>
+      </c>
+      <c r="AE1" s="226">
+        <f>3/(10/2/10000)</f>
+        <v>6000</v>
+      </c>
+      <c r="AF1" s="226">
+        <f>3/(100/2/10000)</f>
+        <v>600</v>
+      </c>
+      <c r="AG1" s="226">
+        <f>3/(1000/2/10000)</f>
+        <v>60</v>
+      </c>
+      <c r="AH1" s="227">
+        <f>3/(5000/2/10000)</f>
+        <v>12</v>
+      </c>
+      <c r="AI1" s="225">
+        <f>3/(1/2/10000)</f>
+        <v>60000</v>
+      </c>
+      <c r="AJ1" s="226">
+        <f>3/(10/2/10000)</f>
+        <v>6000</v>
+      </c>
+      <c r="AK1" s="226">
+        <f>3/(100/2/10000)</f>
+        <v>600</v>
+      </c>
+      <c r="AL1" s="226">
+        <f>3/(1000/2/10000)</f>
+        <v>60</v>
+      </c>
+      <c r="AM1" s="227">
+        <f>3/(5000/2/10000)</f>
+        <v>12</v>
+      </c>
+      <c r="AN1" s="225">
+        <f>3/(1/2/10000)</f>
+        <v>60000</v>
+      </c>
+      <c r="AO1" s="226">
+        <f>3/(10/2/10000)</f>
+        <v>6000</v>
+      </c>
+      <c r="AP1" s="226">
+        <f>3/(100/2/10000)</f>
+        <v>600</v>
+      </c>
+      <c r="AQ1" s="226">
+        <f>3/(1000/2/10000)</f>
+        <v>60</v>
+      </c>
+      <c r="AR1" s="227">
+        <f>3/(5000/2/10000)</f>
+        <v>12</v>
+      </c>
+      <c r="AS1" s="225">
+        <f>3/(1/2/10000)</f>
+        <v>60000</v>
+      </c>
+      <c r="AT1" s="226">
+        <f>3/(10/2/10000)</f>
+        <v>6000</v>
+      </c>
+      <c r="AU1" s="226">
+        <f>3/(100/2/10000)</f>
+        <v>600</v>
+      </c>
+      <c r="AV1" s="226">
+        <f>3/(1000/2/10000)</f>
+        <v>60</v>
+      </c>
+      <c r="AW1" s="227">
+        <f>3/(5000/2/10000)</f>
+        <v>12</v>
+      </c>
+      <c r="AX1" s="225">
+        <f>3/(1/2/10000)</f>
+        <v>60000</v>
+      </c>
+      <c r="AY1" s="226">
+        <f>3/(10/2/10000)</f>
+        <v>6000</v>
+      </c>
+      <c r="AZ1" s="226">
+        <f>3/(100/2/10000)</f>
+        <v>600</v>
+      </c>
+      <c r="BA1" s="226">
+        <f>3/(1000/2/10000)</f>
+        <v>60</v>
+      </c>
+      <c r="BB1" s="227">
+        <f>3/(5000/2/10000)</f>
+        <v>12</v>
+      </c>
+      <c r="BC1" s="225">
+        <f>3/(1/2/10000)</f>
+        <v>60000</v>
+      </c>
+      <c r="BD1" s="226">
+        <f>3/(10/2/10000)</f>
+        <v>6000</v>
+      </c>
+      <c r="BE1" s="226">
+        <f>3/(100/2/10000)</f>
+        <v>600</v>
+      </c>
+      <c r="BF1" s="226">
+        <f>3/(1000/2/10000)</f>
+        <v>60</v>
+      </c>
+      <c r="BG1" s="227">
+        <f>3/(5000/2/10000)</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>874</v>
       </c>
@@ -9894,8 +10436,122 @@
       <c r="U2" s="10" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:22" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V2" s="3" t="s">
+        <v>1017</v>
+      </c>
+      <c r="W2" s="228" t="s">
+        <v>1019</v>
+      </c>
+      <c r="X2" s="238" t="s">
+        <v>1020</v>
+      </c>
+      <c r="Y2" s="228" t="s">
+        <v>1023</v>
+      </c>
+      <c r="Z2" s="229" t="s">
+        <v>1024</v>
+      </c>
+      <c r="AA2" s="230" t="s">
+        <v>1025</v>
+      </c>
+      <c r="AB2" s="230" t="s">
+        <v>1026</v>
+      </c>
+      <c r="AC2" s="231" t="s">
+        <v>1027</v>
+      </c>
+      <c r="AD2" s="228" t="s">
+        <v>1028</v>
+      </c>
+      <c r="AE2" s="229" t="s">
+        <v>1029</v>
+      </c>
+      <c r="AF2" s="230" t="s">
+        <v>1030</v>
+      </c>
+      <c r="AG2" s="230" t="s">
+        <v>1031</v>
+      </c>
+      <c r="AH2" s="231" t="s">
+        <v>1032</v>
+      </c>
+      <c r="AI2" s="228" t="s">
+        <v>1033</v>
+      </c>
+      <c r="AJ2" s="229" t="s">
+        <v>1034</v>
+      </c>
+      <c r="AK2" s="230" t="s">
+        <v>1035</v>
+      </c>
+      <c r="AL2" s="230" t="s">
+        <v>1036</v>
+      </c>
+      <c r="AM2" s="231" t="s">
+        <v>1037</v>
+      </c>
+      <c r="AN2" s="228" t="s">
+        <v>1038</v>
+      </c>
+      <c r="AO2" s="228" t="s">
+        <v>1042</v>
+      </c>
+      <c r="AP2" s="228" t="s">
+        <v>1041</v>
+      </c>
+      <c r="AQ2" s="228" t="s">
+        <v>1040</v>
+      </c>
+      <c r="AR2" s="246" t="s">
+        <v>1039</v>
+      </c>
+      <c r="AS2" s="228" t="s">
+        <v>1043</v>
+      </c>
+      <c r="AT2" s="228" t="s">
+        <v>1044</v>
+      </c>
+      <c r="AU2" s="228" t="s">
+        <v>1045</v>
+      </c>
+      <c r="AV2" s="228" t="s">
+        <v>1046</v>
+      </c>
+      <c r="AW2" s="246" t="s">
+        <v>1047</v>
+      </c>
+      <c r="AX2" s="228" t="s">
+        <v>1048</v>
+      </c>
+      <c r="AY2" s="228" t="s">
+        <v>1049</v>
+      </c>
+      <c r="AZ2" s="228" t="s">
+        <v>1050</v>
+      </c>
+      <c r="BA2" s="228" t="s">
+        <v>1051</v>
+      </c>
+      <c r="BB2" s="246" t="s">
+        <v>1052</v>
+      </c>
+      <c r="BC2" s="228" t="s">
+        <v>1053</v>
+      </c>
+      <c r="BD2" s="228" t="s">
+        <v>1054</v>
+      </c>
+      <c r="BE2" s="228" t="s">
+        <v>1055</v>
+      </c>
+      <c r="BF2" s="228" t="s">
+        <v>1056</v>
+      </c>
+      <c r="BG2" s="246" t="s">
+        <v>1057</v>
+      </c>
+    </row>
+    <row r="3" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="92" t="s">
         <v>875</v>
       </c>
@@ -9923,14 +10579,14 @@
         <f t="shared" si="0"/>
         <v>1.1232000000000001E-2</v>
       </c>
-      <c r="I3" s="49">
+      <c r="I3" s="223">
         <v>6.1159199469419762E-9</v>
       </c>
       <c r="J3" s="49">
-        <f>B22*R3^C22*(D22*S3^E22+F22*T3^G22)</f>
+        <f>C$31*R3^D$31*(E$31*S3^F$31+G$31*T3^H$31)</f>
         <v>2.5940272363739319E-5</v>
       </c>
-      <c r="K3" s="49">
+      <c r="K3" s="223">
         <v>4.1028436240467077</v>
       </c>
       <c r="L3" s="92" t="s">
@@ -9966,8 +10622,95 @@
         <f>'Drop-down lists'!S8</f>
         <v>250000</v>
       </c>
-    </row>
-    <row r="4" spans="1:22" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V3" s="5"/>
+      <c r="W3" s="232">
+        <v>4.5E-11</v>
+      </c>
+      <c r="X3" s="234">
+        <v>41000000</v>
+      </c>
+      <c r="Y3" s="232">
+        <f>$C$31*Y$1^$D$31*($E$31*$S3^$F$31+$G$31*$T3^$H$31)</f>
+        <v>155.40870028092934</v>
+      </c>
+      <c r="Z3" s="233">
+        <f t="shared" ref="Z3:AC8" si="1">$C$31*Z$1^$D$31*($E$31*$S3^$F$31+$G$31*$T3^$H$31)</f>
+        <v>0.85567411853615005</v>
+      </c>
+      <c r="AA3" s="233">
+        <f t="shared" si="1"/>
+        <v>4.7113076411364066E-3</v>
+      </c>
+      <c r="AB3" s="233">
+        <f t="shared" si="1"/>
+        <v>2.5940272363739319E-5</v>
+      </c>
+      <c r="AC3" s="242">
+        <f t="shared" si="1"/>
+        <v>6.8372996136931691E-7</v>
+      </c>
+      <c r="AD3" s="232">
+        <f>$C$32*AD$1^$D$32*($E$32*$S3^$F$32+$G$32*$T3^$H$32)</f>
+        <v>37711318.658650719</v>
+      </c>
+      <c r="AE3" s="233">
+        <f t="shared" ref="AE3:AH3" si="2">$C$32*AE$1^$D$32*($E$32*$S3^$F$32+$G$32*$T3^$H$32)</f>
+        <v>4705.6097784279227</v>
+      </c>
+      <c r="AF3" s="233">
+        <f t="shared" si="2"/>
+        <v>0.58716491956340644</v>
+      </c>
+      <c r="AG3" s="233">
+        <f t="shared" si="2"/>
+        <v>7.3266305324850092E-5</v>
+      </c>
+      <c r="AH3" s="234">
+        <f t="shared" si="2"/>
+        <v>1.3684413214814805E-7</v>
+      </c>
+      <c r="AI3" s="232">
+        <f>$C$34*AI$1^$D$34*($E$34*$S3^$F$34+$G$34*$T3^$H$34)</f>
+        <v>4.3102186815559843E-4</v>
+      </c>
+      <c r="AJ3" s="233">
+        <f t="shared" ref="AJ3:AM8" si="3">$C$34*AJ$1^$D$34*($E$34*$S3^$F$34+$G$34*$T3^$H$34)</f>
+        <v>4.310218681463646E-4</v>
+      </c>
+      <c r="AK3" s="233">
+        <f t="shared" si="3"/>
+        <v>4.3102186813713078E-4</v>
+      </c>
+      <c r="AL3" s="233">
+        <f t="shared" si="3"/>
+        <v>4.3102186812789701E-4</v>
+      </c>
+      <c r="AM3" s="234">
+        <f t="shared" si="3"/>
+        <v>4.3102186812144275E-4</v>
+      </c>
+      <c r="AN3" s="228"/>
+      <c r="AO3" s="229"/>
+      <c r="AP3" s="229"/>
+      <c r="AQ3" s="229"/>
+      <c r="AR3" s="238"/>
+      <c r="AS3" s="228"/>
+      <c r="AT3" s="229"/>
+      <c r="AU3" s="229"/>
+      <c r="AV3" s="229"/>
+      <c r="AW3" s="238"/>
+      <c r="AX3" s="228"/>
+      <c r="AY3" s="229"/>
+      <c r="AZ3" s="229"/>
+      <c r="BA3" s="229"/>
+      <c r="BB3" s="238"/>
+      <c r="BC3" s="228"/>
+      <c r="BD3" s="229"/>
+      <c r="BE3" s="229"/>
+      <c r="BF3" s="229"/>
+      <c r="BG3" s="238"/>
+    </row>
+    <row r="4" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="92" t="s">
         <v>876</v>
       </c>
@@ -9984,7 +10727,7 @@
         <v>843</v>
       </c>
       <c r="F4" s="49">
-        <f t="shared" ref="F4" si="1">24*3600*N4</f>
+        <f t="shared" ref="F4" si="4">24*3600*N4</f>
         <v>8.6399999999999994E-16</v>
       </c>
       <c r="G4" s="49">
@@ -9992,17 +10735,17 @@
         <v>2.3327999999999999E-3</v>
       </c>
       <c r="H4" s="49">
-        <f t="shared" ref="H4" si="2">24*3600*P4</f>
+        <f t="shared" ref="H4" si="5">24*3600*P4</f>
         <v>1.1232000000000001E-2</v>
       </c>
-      <c r="I4" s="49">
+      <c r="I4" s="223">
         <v>5.7460269656489123E-9</v>
       </c>
       <c r="J4" s="49">
-        <f>B22*R4^C22*(D22*S4^E22+F22*T4^G22)</f>
+        <f t="shared" ref="J4:J9" si="6">C$31*R4^D$31*(E$31*S4^F$31+G$31*T4^H$31)</f>
         <v>2.5874138434805292E-5</v>
       </c>
-      <c r="K4" s="49">
+      <c r="K4" s="223">
         <v>2.0582360578320475</v>
       </c>
       <c r="L4" s="92" t="s">
@@ -10024,7 +10767,7 @@
         <v>833</v>
       </c>
       <c r="R4" s="4">
-        <f t="shared" ref="R4:R13" si="3">6/1000*10^4</f>
+        <f t="shared" ref="R4:R13" si="7">6/1000*10^4</f>
         <v>60</v>
       </c>
       <c r="S4" s="4">
@@ -10038,8 +10781,95 @@
         <f>'Drop-down lists'!S5</f>
         <v>670000000</v>
       </c>
-    </row>
-    <row r="5" spans="1:22" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V4" s="5"/>
+      <c r="W4" s="232">
+        <v>4.1000000000000001E-11</v>
+      </c>
+      <c r="X4" s="234">
+        <v>52000000</v>
+      </c>
+      <c r="Y4" s="232">
+        <f t="shared" ref="Y4:Y5" si="8">$C$31*Y$1^$D$31*($E$31*$S4^$F$31+$G$31*$T4^$H$31)</f>
+        <v>155.01249056516417</v>
+      </c>
+      <c r="Z4" s="233">
+        <f t="shared" si="1"/>
+        <v>0.85349260361015189</v>
+      </c>
+      <c r="AA4" s="233">
+        <f t="shared" si="1"/>
+        <v>4.6992963067773738E-3</v>
+      </c>
+      <c r="AB4" s="233">
+        <f t="shared" si="1"/>
+        <v>2.5874138434805292E-5</v>
+      </c>
+      <c r="AC4" s="242">
+        <f t="shared" si="1"/>
+        <v>6.8198681279935548E-7</v>
+      </c>
+      <c r="AD4" s="232">
+        <f t="shared" ref="AD4:AH8" si="9">$C$32*AD$1^$D$32*($E$32*$S4^$F$32+$G$32*$T4^$H$32)</f>
+        <v>2998876.7761381557</v>
+      </c>
+      <c r="AE4" s="233">
+        <f t="shared" si="9"/>
+        <v>374.19916311674814</v>
+      </c>
+      <c r="AF4" s="233">
+        <f t="shared" si="9"/>
+        <v>4.6692486597463598E-2</v>
+      </c>
+      <c r="AG4" s="233">
+        <f t="shared" si="9"/>
+        <v>5.8262778743150289E-6</v>
+      </c>
+      <c r="AH4" s="234">
+        <f t="shared" si="9"/>
+        <v>1.0882109256493047E-8</v>
+      </c>
+      <c r="AI4" s="232">
+        <f t="shared" ref="AI4:AI5" si="10">$C$34*AI$1^$D$34*($E$34*$S4^$F$34+$G$34*$T4^$H$34)</f>
+        <v>3.7172328113988417E-9</v>
+      </c>
+      <c r="AJ4" s="233">
+        <f t="shared" si="3"/>
+        <v>3.7172328113192074E-9</v>
+      </c>
+      <c r="AK4" s="233">
+        <f t="shared" si="3"/>
+        <v>3.7172328112395726E-9</v>
+      </c>
+      <c r="AL4" s="233">
+        <f t="shared" si="3"/>
+        <v>3.7172328111599383E-9</v>
+      </c>
+      <c r="AM4" s="234">
+        <f t="shared" si="3"/>
+        <v>3.7172328111042753E-9</v>
+      </c>
+      <c r="AN4" s="228"/>
+      <c r="AO4" s="229"/>
+      <c r="AP4" s="229"/>
+      <c r="AQ4" s="229"/>
+      <c r="AR4" s="238"/>
+      <c r="AS4" s="228"/>
+      <c r="AT4" s="229"/>
+      <c r="AU4" s="229"/>
+      <c r="AV4" s="229"/>
+      <c r="AW4" s="238"/>
+      <c r="AX4" s="228"/>
+      <c r="AY4" s="229"/>
+      <c r="AZ4" s="229"/>
+      <c r="BA4" s="229"/>
+      <c r="BB4" s="238"/>
+      <c r="BC4" s="228"/>
+      <c r="BD4" s="229"/>
+      <c r="BE4" s="229"/>
+      <c r="BF4" s="229"/>
+      <c r="BG4" s="238"/>
+    </row>
+    <row r="5" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="92" t="s">
         <v>878</v>
       </c>
@@ -10056,7 +10886,7 @@
         <v>843</v>
       </c>
       <c r="F5" s="49">
-        <f t="shared" ref="F5" si="4">24*3600*N5</f>
+        <f t="shared" ref="F5" si="11">24*3600*N5</f>
         <v>8.6399999999999994E-16</v>
       </c>
       <c r="G5" s="49">
@@ -10064,17 +10894,17 @@
         <v>2.3327999999999999E-3</v>
       </c>
       <c r="H5" s="49">
-        <f t="shared" ref="H5" si="5">24*3600*P5</f>
+        <f t="shared" ref="H5" si="12">24*3600*P5</f>
         <v>1.1232000000000001E-2</v>
       </c>
-      <c r="I5" s="49">
+      <c r="I5" s="223">
         <v>0</v>
       </c>
       <c r="J5" s="49">
-        <f>B22*R5^C22*(D22*S5^E22+F22*T5^G22)</f>
-        <v>0</v>
-      </c>
-      <c r="K5" s="49">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="K5" s="223">
         <v>0</v>
       </c>
       <c r="L5" s="92" t="s">
@@ -10096,7 +10926,7 @@
         <v>833</v>
       </c>
       <c r="R5" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>60</v>
       </c>
       <c r="S5" s="4">
@@ -10110,8 +10940,95 @@
         <f>'Drop-down lists'!S10</f>
         <v>482000</v>
       </c>
-    </row>
-    <row r="6" spans="1:22" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V5" s="5"/>
+      <c r="W5" s="232">
+        <v>0</v>
+      </c>
+      <c r="X5" s="234">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="232">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="233">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AA5" s="233">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AB5" s="233">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AC5" s="234">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AD5" s="232">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="AE5" s="233">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="AF5" s="233">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="AG5" s="233">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="AH5" s="234">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="AI5" s="232">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="AJ5" s="233">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AK5" s="233">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AL5" s="233">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AM5" s="234">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AN5" s="228"/>
+      <c r="AO5" s="229"/>
+      <c r="AP5" s="229"/>
+      <c r="AQ5" s="229"/>
+      <c r="AR5" s="238"/>
+      <c r="AS5" s="228"/>
+      <c r="AT5" s="229"/>
+      <c r="AU5" s="229"/>
+      <c r="AV5" s="229"/>
+      <c r="AW5" s="238"/>
+      <c r="AX5" s="228"/>
+      <c r="AY5" s="229"/>
+      <c r="AZ5" s="229"/>
+      <c r="BA5" s="229"/>
+      <c r="BB5" s="238"/>
+      <c r="BC5" s="228"/>
+      <c r="BD5" s="229"/>
+      <c r="BE5" s="229"/>
+      <c r="BF5" s="229"/>
+      <c r="BG5" s="238"/>
+    </row>
+    <row r="6" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="92" t="s">
         <v>879</v>
       </c>
@@ -10133,14 +11050,14 @@
         <v>2.7397260273972601E-2</v>
       </c>
       <c r="H6" s="92"/>
-      <c r="I6" s="49">
+      <c r="I6" s="223">
         <v>2.4622288189195724E-8</v>
       </c>
       <c r="J6" s="49">
-        <f>B22*R6^C22*(D22*S6^E22+F22*T6^G22)</f>
+        <f t="shared" si="6"/>
         <v>5.2601616232617954E-4</v>
       </c>
-      <c r="K6" s="49">
+      <c r="K6" s="223">
         <v>484.38001378128774</v>
       </c>
       <c r="L6" s="92" t="s">
@@ -10156,7 +11073,7 @@
         <v>837</v>
       </c>
       <c r="R6" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>60</v>
       </c>
       <c r="S6" s="4">
@@ -10170,8 +11087,59 @@
         <f>'Drop-down lists'!S8</f>
         <v>250000</v>
       </c>
-    </row>
-    <row r="7" spans="1:22" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V6" s="5"/>
+      <c r="W6" s="232">
+        <v>3.4E-8</v>
+      </c>
+      <c r="X6" s="234">
+        <v>20</v>
+      </c>
+      <c r="Y6" s="232"/>
+      <c r="Z6" s="233"/>
+      <c r="AA6" s="233"/>
+      <c r="AB6" s="243">
+        <f t="shared" si="1"/>
+        <v>5.2601616232617954E-4</v>
+      </c>
+      <c r="AC6" s="234"/>
+      <c r="AD6" s="232"/>
+      <c r="AE6" s="233"/>
+      <c r="AF6" s="233"/>
+      <c r="AG6" s="233">
+        <f t="shared" si="9"/>
+        <v>3.718319691791454E-4</v>
+      </c>
+      <c r="AH6" s="234"/>
+      <c r="AI6" s="232"/>
+      <c r="AJ6" s="233"/>
+      <c r="AK6" s="233"/>
+      <c r="AL6" s="244">
+        <f t="shared" si="3"/>
+        <v>1.4877364519989206E-3</v>
+      </c>
+      <c r="AM6" s="234"/>
+      <c r="AN6" s="228"/>
+      <c r="AO6" s="229"/>
+      <c r="AP6" s="229"/>
+      <c r="AQ6" s="229"/>
+      <c r="AR6" s="238"/>
+      <c r="AS6" s="228"/>
+      <c r="AT6" s="229"/>
+      <c r="AU6" s="229"/>
+      <c r="AV6" s="229"/>
+      <c r="AW6" s="238"/>
+      <c r="AX6" s="228"/>
+      <c r="AY6" s="229"/>
+      <c r="AZ6" s="229"/>
+      <c r="BA6" s="229"/>
+      <c r="BB6" s="238"/>
+      <c r="BC6" s="228"/>
+      <c r="BD6" s="229"/>
+      <c r="BE6" s="229"/>
+      <c r="BF6" s="229"/>
+      <c r="BG6" s="238"/>
+    </row>
+    <row r="7" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="92" t="s">
         <v>880</v>
       </c>
@@ -10189,18 +11157,18 @@
       </c>
       <c r="F7" s="92"/>
       <c r="G7" s="49">
-        <f t="shared" ref="G7:G8" si="6">1/O7</f>
+        <f t="shared" ref="G7:G8" si="13">1/O7</f>
         <v>2.7397260273972603E-3</v>
       </c>
       <c r="H7" s="92"/>
-      <c r="I7" s="49">
+      <c r="I7" s="223">
         <v>8.168155468460269E-18</v>
       </c>
       <c r="J7" s="49">
-        <f>B22*R7^C22*(D22*S7^E22+F22*T7^G22)</f>
+        <f t="shared" si="6"/>
         <v>9.3866225168064443E-9</v>
       </c>
-      <c r="K7" s="49">
+      <c r="K7" s="223">
         <v>0.72562580886925876</v>
       </c>
       <c r="L7" s="92" t="s">
@@ -10216,7 +11184,7 @@
         <v>837</v>
       </c>
       <c r="R7" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>60</v>
       </c>
       <c r="S7" s="4">
@@ -10230,8 +11198,59 @@
         <f>'Drop-down lists'!S9</f>
         <v>38500</v>
       </c>
-    </row>
-    <row r="8" spans="1:22" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V7" s="5"/>
+      <c r="W7" s="232">
+        <v>1.4000000000000001E-20</v>
+      </c>
+      <c r="X7" s="234">
+        <v>0.31</v>
+      </c>
+      <c r="Y7" s="232"/>
+      <c r="Z7" s="233"/>
+      <c r="AA7" s="233"/>
+      <c r="AB7" s="233">
+        <f t="shared" si="1"/>
+        <v>9.3866225168064443E-9</v>
+      </c>
+      <c r="AC7" s="234"/>
+      <c r="AD7" s="232"/>
+      <c r="AE7" s="233"/>
+      <c r="AF7" s="233"/>
+      <c r="AG7" s="243">
+        <f t="shared" si="9"/>
+        <v>1.5713621209990987E-20</v>
+      </c>
+      <c r="AH7" s="234"/>
+      <c r="AI7" s="232"/>
+      <c r="AJ7" s="233"/>
+      <c r="AK7" s="233"/>
+      <c r="AL7" s="244">
+        <f t="shared" si="3"/>
+        <v>3.9741885154506359E-8</v>
+      </c>
+      <c r="AM7" s="234"/>
+      <c r="AN7" s="228"/>
+      <c r="AO7" s="229"/>
+      <c r="AP7" s="229"/>
+      <c r="AQ7" s="229"/>
+      <c r="AR7" s="238"/>
+      <c r="AS7" s="228"/>
+      <c r="AT7" s="229"/>
+      <c r="AU7" s="229"/>
+      <c r="AV7" s="229"/>
+      <c r="AW7" s="238"/>
+      <c r="AX7" s="228"/>
+      <c r="AY7" s="229"/>
+      <c r="AZ7" s="229"/>
+      <c r="BA7" s="229"/>
+      <c r="BB7" s="238"/>
+      <c r="BC7" s="228"/>
+      <c r="BD7" s="229"/>
+      <c r="BE7" s="229"/>
+      <c r="BF7" s="229"/>
+      <c r="BG7" s="238"/>
+    </row>
+    <row r="8" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="92" t="s">
         <v>881</v>
       </c>
@@ -10249,18 +11268,18 @@
       </c>
       <c r="F8" s="92"/>
       <c r="G8" s="49">
+        <f t="shared" si="13"/>
+        <v>2.7397260273972603E-3</v>
+      </c>
+      <c r="H8" s="92"/>
+      <c r="I8" s="223">
+        <v>0</v>
+      </c>
+      <c r="J8" s="49">
         <f t="shared" si="6"/>
-        <v>2.7397260273972603E-3</v>
-      </c>
-      <c r="H8" s="92"/>
-      <c r="I8" s="49">
-        <v>0</v>
-      </c>
-      <c r="J8" s="49">
-        <f>B22*R8^C22*(D22*S8^E22+F22*T8^G22)</f>
-        <v>0</v>
-      </c>
-      <c r="K8" s="49">
+        <v>0</v>
+      </c>
+      <c r="K8" s="223">
         <v>0</v>
       </c>
       <c r="L8" s="92" t="s">
@@ -10276,7 +11295,7 @@
         <v>837</v>
       </c>
       <c r="R8" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>60</v>
       </c>
       <c r="S8" s="4">
@@ -10290,8 +11309,54 @@
         <f>'Drop-down lists'!S10</f>
         <v>482000</v>
       </c>
-    </row>
-    <row r="9" spans="1:22" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W8" s="228"/>
+      <c r="X8" s="238"/>
+      <c r="Y8" s="232"/>
+      <c r="Z8" s="233"/>
+      <c r="AA8" s="233"/>
+      <c r="AB8" s="233">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AC8" s="234"/>
+      <c r="AD8" s="232"/>
+      <c r="AE8" s="233"/>
+      <c r="AF8" s="233"/>
+      <c r="AG8" s="233">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="AH8" s="234"/>
+      <c r="AI8" s="232"/>
+      <c r="AJ8" s="233"/>
+      <c r="AK8" s="233"/>
+      <c r="AL8" s="233">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AM8" s="234"/>
+      <c r="AN8" s="228"/>
+      <c r="AO8" s="229"/>
+      <c r="AP8" s="229"/>
+      <c r="AQ8" s="229"/>
+      <c r="AR8" s="238"/>
+      <c r="AS8" s="228"/>
+      <c r="AT8" s="229"/>
+      <c r="AU8" s="229"/>
+      <c r="AV8" s="229"/>
+      <c r="AW8" s="238"/>
+      <c r="AX8" s="228"/>
+      <c r="AY8" s="229"/>
+      <c r="AZ8" s="229"/>
+      <c r="BA8" s="229"/>
+      <c r="BB8" s="238"/>
+      <c r="BC8" s="228"/>
+      <c r="BD8" s="229"/>
+      <c r="BE8" s="229"/>
+      <c r="BF8" s="229"/>
+      <c r="BG8" s="238"/>
+    </row>
+    <row r="9" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="92" t="s">
         <v>882</v>
       </c>
@@ -10313,14 +11378,14 @@
         <v>5.4821917808219178E-5</v>
       </c>
       <c r="H9" s="92"/>
-      <c r="I9" s="49">
+      <c r="I9" s="223">
         <v>5.6645194590916446E-8</v>
       </c>
       <c r="J9" s="49">
-        <f>B22*R9^C22*(D22*S9^E22+F22*T9^G22)</f>
+        <f>C$31*R9^D$31*(E$31*S9^F$31+G$31*T9^H$31)</f>
         <v>1.6521772091595942E-4</v>
       </c>
-      <c r="K9" s="49">
+      <c r="K9" s="223">
         <v>3.5299794836927361</v>
       </c>
       <c r="L9" s="92" t="s">
@@ -10356,8 +11421,45 @@
       <c r="V9" s="4" t="s">
         <v>1005</v>
       </c>
-    </row>
-    <row r="10" spans="1:22" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W9" s="228"/>
+      <c r="X9" s="238"/>
+      <c r="Y9" s="232"/>
+      <c r="Z9" s="233"/>
+      <c r="AA9" s="233"/>
+      <c r="AB9" s="233"/>
+      <c r="AC9" s="234"/>
+      <c r="AD9" s="228"/>
+      <c r="AE9" s="229"/>
+      <c r="AF9" s="229"/>
+      <c r="AG9" s="229"/>
+      <c r="AH9" s="238"/>
+      <c r="AI9" s="228"/>
+      <c r="AJ9" s="229"/>
+      <c r="AK9" s="229"/>
+      <c r="AL9" s="229"/>
+      <c r="AM9" s="238"/>
+      <c r="AN9" s="228"/>
+      <c r="AO9" s="229"/>
+      <c r="AP9" s="229"/>
+      <c r="AQ9" s="229"/>
+      <c r="AR9" s="238"/>
+      <c r="AS9" s="228"/>
+      <c r="AT9" s="229"/>
+      <c r="AU9" s="229"/>
+      <c r="AV9" s="229"/>
+      <c r="AW9" s="238"/>
+      <c r="AX9" s="228"/>
+      <c r="AY9" s="229"/>
+      <c r="AZ9" s="229"/>
+      <c r="BA9" s="229"/>
+      <c r="BB9" s="238"/>
+      <c r="BC9" s="228"/>
+      <c r="BD9" s="229"/>
+      <c r="BE9" s="229"/>
+      <c r="BF9" s="229"/>
+      <c r="BG9" s="238"/>
+    </row>
+    <row r="10" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="92" t="s">
         <v>882</v>
       </c>
@@ -10379,14 +11481,14 @@
         <v>5.1041095890410963E-6</v>
       </c>
       <c r="H10" s="92"/>
-      <c r="I10" s="49">
+      <c r="I10" s="223">
         <v>3.1438231723910843E-8</v>
       </c>
       <c r="J10" s="49">
-        <f>B22*R10^C22*(D22*S10^E22+F22*T10^G22)</f>
+        <f>C$31*R10^D$31*(E$31*S10^F$31+G$31*T10^H$31)</f>
         <v>1.6348682453580125E-4</v>
       </c>
-      <c r="K10" s="49">
+      <c r="K10" s="223">
         <v>3.300948856770983</v>
       </c>
       <c r="L10" s="92" t="s">
@@ -10421,8 +11523,45 @@
       <c r="V10" s="4" t="s">
         <v>1006</v>
       </c>
-    </row>
-    <row r="11" spans="1:22" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W10" s="239"/>
+      <c r="X10" s="241"/>
+      <c r="Y10" s="235"/>
+      <c r="Z10" s="236"/>
+      <c r="AA10" s="236"/>
+      <c r="AB10" s="236"/>
+      <c r="AC10" s="237"/>
+      <c r="AD10" s="239"/>
+      <c r="AE10" s="240"/>
+      <c r="AF10" s="240"/>
+      <c r="AG10" s="240"/>
+      <c r="AH10" s="241"/>
+      <c r="AI10" s="239"/>
+      <c r="AJ10" s="240"/>
+      <c r="AK10" s="240"/>
+      <c r="AL10" s="240"/>
+      <c r="AM10" s="241"/>
+      <c r="AN10" s="239"/>
+      <c r="AO10" s="240"/>
+      <c r="AP10" s="240"/>
+      <c r="AQ10" s="240"/>
+      <c r="AR10" s="241"/>
+      <c r="AS10" s="239"/>
+      <c r="AT10" s="240"/>
+      <c r="AU10" s="240"/>
+      <c r="AV10" s="240"/>
+      <c r="AW10" s="241"/>
+      <c r="AX10" s="239"/>
+      <c r="AY10" s="240"/>
+      <c r="AZ10" s="240"/>
+      <c r="BA10" s="240"/>
+      <c r="BB10" s="241"/>
+      <c r="BC10" s="239"/>
+      <c r="BD10" s="240"/>
+      <c r="BE10" s="240"/>
+      <c r="BF10" s="240"/>
+      <c r="BG10" s="241"/>
+    </row>
+    <row r="11" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="43" t="s">
         <v>877</v>
       </c>
@@ -10439,25 +11578,25 @@
         <v>843</v>
       </c>
       <c r="F11" s="42">
-        <f t="shared" ref="F11:H12" si="7">24*3600*N11</f>
+        <f t="shared" ref="F11:H12" si="14">24*3600*N11</f>
         <v>8.6399999999999994E-16</v>
       </c>
       <c r="G11" s="42">
-        <f t="shared" si="7"/>
+        <f t="shared" si="14"/>
         <v>8.6400000000000003E-6</v>
       </c>
       <c r="H11" s="42">
-        <f t="shared" si="7"/>
+        <f t="shared" si="14"/>
         <v>1.728E-4</v>
       </c>
-      <c r="I11" s="42">
+      <c r="I11" s="223">
         <v>2.4029970147489989E-4</v>
       </c>
       <c r="J11" s="42">
-        <f>B23*R11^C23*(D23*S11^E23+F23*U11^G23)</f>
+        <f>C$44*R11^D$44*(E$44*S11^F$44+G$44*U11^H$44)</f>
         <v>5.3195434885788091E-4</v>
       </c>
-      <c r="K11" s="42">
+      <c r="K11" s="223">
         <v>3.1319232337502488E-3</v>
       </c>
       <c r="L11" s="43" t="s">
@@ -10479,7 +11618,7 @@
         <v>833</v>
       </c>
       <c r="R11" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>60</v>
       </c>
       <c r="S11" s="4">
@@ -10492,8 +11631,140 @@
       <c r="U11" s="5">
         <v>250000</v>
       </c>
-    </row>
-    <row r="12" spans="1:22" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V11" s="5"/>
+      <c r="W11" s="232">
+        <v>4.8500000000000002E-6</v>
+      </c>
+      <c r="X11" s="234">
+        <v>3.69</v>
+      </c>
+      <c r="Y11" s="247">
+        <f>$C$44*Y$1^$D$44*($E$44*$S11^$F$44+$G$44*$U11^$H$44)</f>
+        <v>5.8483955247378371E-4</v>
+      </c>
+      <c r="Z11" s="247">
+        <f t="shared" ref="Z11:AC16" si="15">$C$44*Z$1^$D$44*($E$44*$S11^$F$44+$G$44*$U11^$H$44)</f>
+        <v>5.6665137287759701E-4</v>
+      </c>
+      <c r="AA11" s="247">
+        <f t="shared" si="15"/>
+        <v>5.4902883538893144E-4</v>
+      </c>
+      <c r="AB11" s="247">
+        <f t="shared" si="15"/>
+        <v>5.3195434885788091E-4</v>
+      </c>
+      <c r="AC11" s="247">
+        <f t="shared" si="15"/>
+        <v>5.2033608199586944E-4</v>
+      </c>
+      <c r="AD11" s="247">
+        <f>$C$45*AD$1^$D$45*($E$45*$S11^$F$45+$G$45*$U11^$H$45)</f>
+        <v>7.038593464767487E-4</v>
+      </c>
+      <c r="AE11" s="247">
+        <f t="shared" ref="AE11:AH16" si="16">$C$45*AE$1^$D$45*($E$45*$S11^$F$45+$G$45*$U11^$H$45)</f>
+        <v>4.0196986091351058E-4</v>
+      </c>
+      <c r="AF11" s="247">
+        <f t="shared" si="16"/>
+        <v>2.2956258220002855E-4</v>
+      </c>
+      <c r="AG11" s="247">
+        <f t="shared" si="16"/>
+        <v>1.3110181700334939E-4</v>
+      </c>
+      <c r="AH11" s="247">
+        <f t="shared" si="16"/>
+        <v>8.8624669307802605E-5</v>
+      </c>
+      <c r="AI11" s="247"/>
+      <c r="AJ11" s="248"/>
+      <c r="AK11" s="248"/>
+      <c r="AL11" s="248"/>
+      <c r="AM11" s="256"/>
+      <c r="AN11" s="247">
+        <f>$C$41*AN$1^$D$41*($E$41*$S11^$F$41+$G$41*$U11^$H$41)</f>
+        <v>1.01791542719624E-4</v>
+      </c>
+      <c r="AO11" s="247">
+        <f t="shared" ref="AO11:AR16" si="17">$C$41*AO$1^$D$41*($E$41*$S11^$F$41+$G$41*$U11^$H$41)</f>
+        <v>1.0179154271175244E-4</v>
+      </c>
+      <c r="AP11" s="247">
+        <f t="shared" si="17"/>
+        <v>1.0179154270388089E-4</v>
+      </c>
+      <c r="AQ11" s="247">
+        <f t="shared" si="17"/>
+        <v>1.0179154269600934E-4</v>
+      </c>
+      <c r="AR11" s="247">
+        <f t="shared" si="17"/>
+        <v>1.0179154269050733E-4</v>
+      </c>
+      <c r="AS11" s="247">
+        <f>$C$42*AS$1^$D$42*($E$42*$S11^$F$42+$G$42*$U11^$H$42)</f>
+        <v>1.8011813921940556E-4</v>
+      </c>
+      <c r="AT11" s="247">
+        <f t="shared" ref="AT11:AW16" si="18">$C$42*AT$1^$D$42*($E$42*$S11^$F$42+$G$42*$U11^$H$42)</f>
+        <v>1.8011813921919821E-4</v>
+      </c>
+      <c r="AU11" s="247">
+        <f t="shared" si="18"/>
+        <v>1.8011813921899083E-4</v>
+      </c>
+      <c r="AV11" s="247">
+        <f t="shared" si="18"/>
+        <v>1.8011813921878345E-4</v>
+      </c>
+      <c r="AW11" s="247">
+        <f t="shared" si="18"/>
+        <v>1.8011813921863849E-4</v>
+      </c>
+      <c r="AX11" s="247">
+        <f>$C$43*AX$1^$D$43*($E$43*$S11^$F$43+$G$43*$U11^$H$43)</f>
+        <v>0.46869829319969997</v>
+      </c>
+      <c r="AY11" s="247">
+        <f t="shared" ref="AY11:BB16" si="19">$C$43*AY$1^$D$43*($E$43*$S11^$F$43+$G$43*$U11^$H$43)</f>
+        <v>2.1049718421291577E-2</v>
+      </c>
+      <c r="AZ11" s="247">
+        <f t="shared" si="19"/>
+        <v>9.4536432507739607E-4</v>
+      </c>
+      <c r="BA11" s="247">
+        <f t="shared" si="19"/>
+        <v>4.2457276113729818E-5</v>
+      </c>
+      <c r="BB11" s="247">
+        <f t="shared" si="19"/>
+        <v>4.8527424424727678E-6</v>
+      </c>
+      <c r="BC11" s="247">
+        <f>$C$46*BC$1^$D$46*($E$46*$S11^$F$46+$G$46*$U11^$H$46)</f>
+        <v>6.0533189871791272E-2</v>
+      </c>
+      <c r="BD11" s="247">
+        <f t="shared" ref="BD11:BG16" si="20">$C$46*BD$1^$D$46*($E$46*$S11^$F$46+$G$46*$U11^$H$46)</f>
+        <v>9.7953010729097383E-3</v>
+      </c>
+      <c r="BE11" s="247">
+        <f t="shared" si="20"/>
+        <v>1.5850465391327238E-3</v>
+      </c>
+      <c r="BF11" s="247">
+        <f t="shared" si="20"/>
+        <v>2.5648752524462331E-4</v>
+      </c>
+      <c r="BG11" s="247">
+        <f t="shared" si="20"/>
+        <v>7.1812146657836885E-5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="43" t="s">
         <v>876</v>
       </c>
@@ -10510,25 +11781,25 @@
         <v>843</v>
       </c>
       <c r="F12" s="42">
-        <f t="shared" si="7"/>
+        <f t="shared" si="14"/>
         <v>8.6399999999999994E-16</v>
       </c>
       <c r="G12" s="42">
-        <f t="shared" si="7"/>
+        <f t="shared" si="14"/>
         <v>2.5919999999999999E-6</v>
       </c>
       <c r="H12" s="42">
-        <f t="shared" si="7"/>
+        <f t="shared" si="14"/>
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="I12" s="42">
+      <c r="I12" s="223">
         <v>1.460412381613051E-4</v>
       </c>
       <c r="J12" s="42">
-        <f>B23*R12^C23*(D23*S12^E23+F23*U12^G23)</f>
+        <f t="shared" ref="J12:J17" si="21">C$44*R12^D$44*(E$44*S12^F$44+G$44*U12^H$44)</f>
         <v>7.6984184029519817E-4</v>
       </c>
-      <c r="K12" s="42">
+      <c r="K12" s="223">
         <v>6.993295207079777E-3</v>
       </c>
       <c r="L12" s="43" t="s">
@@ -10550,7 +11821,7 @@
         <v>833</v>
       </c>
       <c r="R12" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>60</v>
       </c>
       <c r="S12" s="4">
@@ -10563,8 +11834,140 @@
       <c r="U12" s="5">
         <v>670000000</v>
       </c>
-    </row>
-    <row r="13" spans="1:22" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V12" s="5"/>
+      <c r="W12" s="232">
+        <v>3.98E-6</v>
+      </c>
+      <c r="X12" s="234">
+        <v>6.44</v>
+      </c>
+      <c r="Y12" s="247">
+        <f>$C$44*Y$1^$D$44*($E$44*$S12^$F$44+$G$44*$U12^$H$44)</f>
+        <v>8.4637705908505341E-4</v>
+      </c>
+      <c r="Z12" s="247">
+        <f t="shared" si="15"/>
+        <v>8.2005521082493356E-4</v>
+      </c>
+      <c r="AA12" s="247">
+        <f t="shared" si="15"/>
+        <v>7.9455195717154559E-4</v>
+      </c>
+      <c r="AB12" s="247">
+        <f t="shared" si="15"/>
+        <v>7.6984184029519817E-4</v>
+      </c>
+      <c r="AC12" s="247">
+        <f t="shared" si="15"/>
+        <v>7.5302793894953745E-4</v>
+      </c>
+      <c r="AD12" s="247">
+        <f t="shared" ref="AD12:AD13" si="22">$C$45*AD$1^$D$45*($E$45*$S12^$F$45+$G$45*$U12^$H$45)</f>
+        <v>5.9186923304184848E-3</v>
+      </c>
+      <c r="AE12" s="247">
+        <f t="shared" si="16"/>
+        <v>3.3801297727411401E-3</v>
+      </c>
+      <c r="AF12" s="247">
+        <f t="shared" si="16"/>
+        <v>1.9303718866838342E-3</v>
+      </c>
+      <c r="AG12" s="247">
+        <f t="shared" si="16"/>
+        <v>1.1024238332356712E-3</v>
+      </c>
+      <c r="AH12" s="247">
+        <f t="shared" si="16"/>
+        <v>7.4523717436391745E-4</v>
+      </c>
+      <c r="AI12" s="232"/>
+      <c r="AJ12" s="233"/>
+      <c r="AK12" s="233"/>
+      <c r="AL12" s="233"/>
+      <c r="AM12" s="234"/>
+      <c r="AN12" s="247">
+        <f>$C$41*AN$1^$D$41*($E$41*$S12^$F$41+$G$41*$U12^$H$41)</f>
+        <v>3.2713613604297924E-4</v>
+      </c>
+      <c r="AO12" s="247">
+        <f t="shared" si="17"/>
+        <v>3.2713613601768177E-4</v>
+      </c>
+      <c r="AP12" s="247">
+        <f t="shared" si="17"/>
+        <v>3.271361359923843E-4</v>
+      </c>
+      <c r="AQ12" s="247">
+        <f t="shared" si="17"/>
+        <v>3.2713613596708677E-4</v>
+      </c>
+      <c r="AR12" s="247">
+        <f t="shared" si="17"/>
+        <v>3.2713613594940457E-4</v>
+      </c>
+      <c r="AS12" s="247">
+        <f t="shared" ref="AS12:AS13" si="23">$C$42*AS$1^$D$42*($E$42*$S12^$F$42+$G$42*$U12^$H$42)</f>
+        <v>9.5179530878247546E-4</v>
+      </c>
+      <c r="AT12" s="247">
+        <f t="shared" si="18"/>
+        <v>9.5179530878137977E-4</v>
+      </c>
+      <c r="AU12" s="247">
+        <f t="shared" si="18"/>
+        <v>9.5179530878028397E-4</v>
+      </c>
+      <c r="AV12" s="247">
+        <f t="shared" si="18"/>
+        <v>9.5179530877918795E-4</v>
+      </c>
+      <c r="AW12" s="247">
+        <f t="shared" si="18"/>
+        <v>9.5179530877842207E-4</v>
+      </c>
+      <c r="AX12" s="247">
+        <f t="shared" ref="AX12:AX13" si="24">$C$43*AX$1^$D$43*($E$43*$S12^$F$43+$G$43*$U12^$H$43)</f>
+        <v>0.38430457321899991</v>
+      </c>
+      <c r="AY12" s="247">
+        <f t="shared" si="19"/>
+        <v>1.7259510375105754E-2</v>
+      </c>
+      <c r="AZ12" s="247">
+        <f t="shared" si="19"/>
+        <v>7.7514221569938754E-4</v>
+      </c>
+      <c r="BA12" s="247">
+        <f t="shared" si="19"/>
+        <v>3.4812427554491084E-5</v>
+      </c>
+      <c r="BB12" s="247">
+        <f t="shared" si="19"/>
+        <v>3.978958618698504E-6</v>
+      </c>
+      <c r="BC12" s="247">
+        <f t="shared" ref="BC12:BC13" si="25">$C$46*BC$1^$D$46*($E$46*$S12^$F$46+$G$46*$U12^$H$46)</f>
+        <v>0.10974080370111601</v>
+      </c>
+      <c r="BD12" s="247">
+        <f t="shared" si="20"/>
+        <v>1.7757931054223977E-2</v>
+      </c>
+      <c r="BE12" s="247">
+        <f t="shared" si="20"/>
+        <v>2.8735356830940167E-3</v>
+      </c>
+      <c r="BF12" s="247">
+        <f t="shared" si="20"/>
+        <v>4.6498701322812556E-4</v>
+      </c>
+      <c r="BG12" s="247">
+        <f t="shared" si="20"/>
+        <v>1.3018845870215544E-4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="43" t="s">
         <v>878</v>
       </c>
@@ -10581,7 +11984,7 @@
         <v>843</v>
       </c>
       <c r="F13" s="42">
-        <f t="shared" ref="F13" si="8">24*3600*N13</f>
+        <f t="shared" ref="F13" si="26">24*3600*N13</f>
         <v>8.6399999999999994E-16</v>
       </c>
       <c r="G13" s="42">
@@ -10589,17 +11992,17 @@
         <v>2.5919999999999999E-6</v>
       </c>
       <c r="H13" s="42">
-        <f t="shared" ref="H13" si="9">24*3600*P13</f>
+        <f t="shared" ref="H13" si="27">24*3600*P13</f>
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="I13" s="42">
+      <c r="I13" s="223">
         <v>9.7418189261740999E-6</v>
       </c>
       <c r="J13" s="42">
-        <f>B23*R13^C23*(D23*S13^E23+F23*U13^G23)</f>
+        <f>C$44*R13^D$44*(E$44*S13^F$44+G$44*U13^H$44)</f>
         <v>3.0587714365284148E-5</v>
       </c>
-      <c r="K13" s="42">
+      <c r="K13" s="223">
         <v>1.2383002084715778E-4</v>
       </c>
       <c r="L13" s="43" t="s">
@@ -10621,7 +12024,7 @@
         <v>833</v>
       </c>
       <c r="R13" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>60</v>
       </c>
       <c r="S13" s="4">
@@ -10634,8 +12037,140 @@
       <c r="U13" s="5">
         <v>482000</v>
       </c>
-    </row>
-    <row r="14" spans="1:22" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V13" s="5"/>
+      <c r="W13" s="232">
+        <v>3.5800000000000003E-8</v>
+      </c>
+      <c r="X13" s="234">
+        <v>3.65</v>
+      </c>
+      <c r="Y13" s="247">
+        <f t="shared" ref="Y12:Y13" si="28">$C$44*Y$1^$D$44*($E$44*$S13^$F$44+$G$44*$U13^$H$44)</f>
+        <v>3.3628647305913803E-5</v>
+      </c>
+      <c r="Z13" s="247">
+        <f t="shared" si="15"/>
+        <v>3.2582815377841188E-5</v>
+      </c>
+      <c r="AA13" s="247">
+        <f t="shared" si="15"/>
+        <v>3.1569508231744662E-5</v>
+      </c>
+      <c r="AB13" s="247">
+        <f t="shared" si="15"/>
+        <v>3.0587714365284148E-5</v>
+      </c>
+      <c r="AC13" s="247">
+        <f t="shared" si="15"/>
+        <v>2.991965661003155E-5</v>
+      </c>
+      <c r="AD13" s="247">
+        <f t="shared" si="22"/>
+        <v>1.6321338455446772E-4</v>
+      </c>
+      <c r="AE13" s="247">
+        <f t="shared" si="16"/>
+        <v>9.3210187258271996E-5</v>
+      </c>
+      <c r="AF13" s="247">
+        <f t="shared" si="16"/>
+        <v>5.3231780178069385E-5</v>
+      </c>
+      <c r="AG13" s="247">
+        <f t="shared" si="16"/>
+        <v>3.0400351123367466E-5</v>
+      </c>
+      <c r="AH13" s="247">
+        <f t="shared" si="16"/>
+        <v>2.0550600493055679E-5</v>
+      </c>
+      <c r="AI13" s="232"/>
+      <c r="AJ13" s="233"/>
+      <c r="AK13" s="233"/>
+      <c r="AL13" s="233"/>
+      <c r="AM13" s="234"/>
+      <c r="AN13" s="247">
+        <f t="shared" ref="AN12:AN13" si="29">$C$41*AN$1^$D$41*($E$41*$S13^$F$41+$G$41*$U13^$H$41)</f>
+        <v>6.593297756474098E-5</v>
+      </c>
+      <c r="AO13" s="247">
+        <f t="shared" si="17"/>
+        <v>6.593297755964237E-5</v>
+      </c>
+      <c r="AP13" s="247">
+        <f t="shared" si="17"/>
+        <v>6.5932977554543761E-5</v>
+      </c>
+      <c r="AQ13" s="247">
+        <f t="shared" si="17"/>
+        <v>6.5932977549445151E-5</v>
+      </c>
+      <c r="AR13" s="247">
+        <f t="shared" si="17"/>
+        <v>6.5932977545881378E-5</v>
+      </c>
+      <c r="AS13" s="247">
+        <f t="shared" si="23"/>
+        <v>8.0391222994992016E-5</v>
+      </c>
+      <c r="AT13" s="247">
+        <f t="shared" si="18"/>
+        <v>8.0391222994899466E-5</v>
+      </c>
+      <c r="AU13" s="247">
+        <f t="shared" si="18"/>
+        <v>8.0391222994806902E-5</v>
+      </c>
+      <c r="AV13" s="247">
+        <f t="shared" si="18"/>
+        <v>8.0391222994714338E-5</v>
+      </c>
+      <c r="AW13" s="247">
+        <f t="shared" si="18"/>
+        <v>8.0391222994649652E-5</v>
+      </c>
+      <c r="AX13" s="247">
+        <f t="shared" si="24"/>
+        <v>3.4596730786513644E-3</v>
+      </c>
+      <c r="AY13" s="247">
+        <f t="shared" si="19"/>
+        <v>1.5537744683935791E-4</v>
+      </c>
+      <c r="AZ13" s="247">
+        <f t="shared" si="19"/>
+        <v>6.9781596230267172E-6</v>
+      </c>
+      <c r="BA13" s="247">
+        <f t="shared" si="19"/>
+        <v>3.1339626641429535E-7</v>
+      </c>
+      <c r="BB13" s="247">
+        <f>$C$43*BB$1^$D$43*($E$43*$S13^$F$43+$G$43*$U13^$H$43)</f>
+        <v>3.5820276347152378E-8</v>
+      </c>
+      <c r="BC13" s="247">
+        <f t="shared" si="25"/>
+        <v>6.2195509415561311E-2</v>
+      </c>
+      <c r="BD13" s="247">
+        <f t="shared" si="20"/>
+        <v>1.0064292686355131E-2</v>
+      </c>
+      <c r="BE13" s="247">
+        <f t="shared" si="20"/>
+        <v>1.6285739634327809E-3</v>
+      </c>
+      <c r="BF13" s="247">
+        <f t="shared" si="20"/>
+        <v>2.635310038197716E-4</v>
+      </c>
+      <c r="BG13" s="247">
+        <f t="shared" si="20"/>
+        <v>7.3784200916372363E-5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="43" t="s">
         <v>879</v>
       </c>
@@ -10657,14 +12192,14 @@
         <v>1.3862943611198905E-4</v>
       </c>
       <c r="H14" s="43"/>
-      <c r="I14" s="42">
+      <c r="I14" s="223">
         <v>2.419391281190053E-4</v>
       </c>
       <c r="J14" s="42">
-        <f>B23*R14^C23*(D23*S14^E23+F23*U14^G23)</f>
+        <f t="shared" si="21"/>
         <v>5.3195434885788091E-4</v>
       </c>
-      <c r="K14" s="42">
+      <c r="K14" s="223">
         <v>2.9859124561264329E-3</v>
       </c>
       <c r="L14" s="43" t="s">
@@ -10680,7 +12215,7 @@
         <v>838</v>
       </c>
       <c r="R14" s="4">
-        <f t="shared" ref="R14:R16" si="10">6/1000*10^4</f>
+        <f t="shared" ref="R14:R16" si="30">6/1000*10^4</f>
         <v>60</v>
       </c>
       <c r="S14" s="4">
@@ -10694,8 +12229,68 @@
         <f>'Drop-down lists'!S8</f>
         <v>250000</v>
       </c>
-    </row>
-    <row r="15" spans="1:22" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V14" s="5"/>
+      <c r="W14" s="232">
+        <v>4.2500000000000003E-5</v>
+      </c>
+      <c r="X14" s="234">
+        <v>2.99E-3</v>
+      </c>
+      <c r="Y14" s="232"/>
+      <c r="Z14" s="233"/>
+      <c r="AA14" s="233"/>
+      <c r="AB14" s="247">
+        <f t="shared" si="15"/>
+        <v>5.3195434885788091E-4</v>
+      </c>
+      <c r="AC14" s="245"/>
+      <c r="AD14" s="232"/>
+      <c r="AE14" s="233"/>
+      <c r="AF14" s="233"/>
+      <c r="AG14" s="247">
+        <f t="shared" si="16"/>
+        <v>1.3110181700334939E-4</v>
+      </c>
+      <c r="AH14" s="234"/>
+      <c r="AI14" s="232"/>
+      <c r="AJ14" s="233"/>
+      <c r="AK14" s="233"/>
+      <c r="AL14" s="233"/>
+      <c r="AM14" s="234"/>
+      <c r="AN14" s="232"/>
+      <c r="AO14" s="233"/>
+      <c r="AP14" s="233"/>
+      <c r="AQ14" s="247">
+        <f t="shared" si="17"/>
+        <v>1.0179154269600934E-4</v>
+      </c>
+      <c r="AR14" s="234"/>
+      <c r="AS14" s="232"/>
+      <c r="AT14" s="233"/>
+      <c r="AU14" s="233"/>
+      <c r="AV14" s="247">
+        <f t="shared" si="18"/>
+        <v>1.8011813921878345E-4</v>
+      </c>
+      <c r="AW14" s="234"/>
+      <c r="AX14" s="232"/>
+      <c r="AY14" s="233"/>
+      <c r="AZ14" s="233"/>
+      <c r="BA14" s="247">
+        <f t="shared" si="19"/>
+        <v>4.2457276113729818E-5</v>
+      </c>
+      <c r="BB14" s="234"/>
+      <c r="BC14" s="232"/>
+      <c r="BD14" s="233"/>
+      <c r="BE14" s="233"/>
+      <c r="BF14" s="247">
+        <f t="shared" si="20"/>
+        <v>2.5648752524462331E-4</v>
+      </c>
+      <c r="BG14" s="234"/>
+    </row>
+    <row r="15" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="43" t="s">
         <v>880</v>
       </c>
@@ -10713,18 +12308,18 @@
       </c>
       <c r="F15" s="43"/>
       <c r="G15" s="42">
-        <f t="shared" ref="G15:G16" si="11">LN(2)/O15</f>
+        <f t="shared" ref="G15:G16" si="31">LN(2)/O15</f>
         <v>1.3862943611198905E-4</v>
       </c>
       <c r="H15" s="43"/>
-      <c r="I15" s="42">
+      <c r="I15" s="223">
         <v>3.9221793756292774E-6</v>
       </c>
       <c r="J15" s="42">
-        <f>B23*R15^C23*(D23*S15^E23+F23*U15^G23)</f>
+        <f t="shared" si="21"/>
         <v>1.0006772720094461E-5</v>
       </c>
-      <c r="K15" s="42">
+      <c r="K15" s="223">
         <v>3.0901034205704649E-5</v>
       </c>
       <c r="L15" s="43" t="s">
@@ -10740,7 +12335,7 @@
         <v>838</v>
       </c>
       <c r="R15" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="30"/>
         <v>60</v>
       </c>
       <c r="S15" s="4">
@@ -10754,8 +12349,68 @@
         <f>'Drop-down lists'!S9</f>
         <v>38500</v>
       </c>
-    </row>
-    <row r="16" spans="1:22" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V15" s="5"/>
+      <c r="W15" s="5">
+        <v>6.0500000000000006E-8</v>
+      </c>
+      <c r="X15" s="245">
+        <v>9.6599999999999995E-4</v>
+      </c>
+      <c r="Y15" s="232"/>
+      <c r="Z15" s="233"/>
+      <c r="AA15" s="233"/>
+      <c r="AB15" s="247">
+        <f t="shared" si="15"/>
+        <v>1.0006772720094461E-5</v>
+      </c>
+      <c r="AC15" s="245"/>
+      <c r="AD15" s="232"/>
+      <c r="AE15" s="233"/>
+      <c r="AF15" s="233"/>
+      <c r="AG15" s="247">
+        <f t="shared" si="16"/>
+        <v>8.6783150312938988E-6</v>
+      </c>
+      <c r="AH15" s="234"/>
+      <c r="AI15" s="232"/>
+      <c r="AJ15" s="233"/>
+      <c r="AK15" s="233"/>
+      <c r="AL15" s="233"/>
+      <c r="AM15" s="234"/>
+      <c r="AN15" s="232"/>
+      <c r="AO15" s="233"/>
+      <c r="AP15" s="233"/>
+      <c r="AQ15" s="247">
+        <f t="shared" si="17"/>
+        <v>3.8149484781896284E-5</v>
+      </c>
+      <c r="AR15" s="234"/>
+      <c r="AS15" s="232"/>
+      <c r="AT15" s="233"/>
+      <c r="AU15" s="233"/>
+      <c r="AV15" s="247">
+        <f t="shared" si="18"/>
+        <v>3.5442563194169012E-5</v>
+      </c>
+      <c r="AW15" s="234"/>
+      <c r="AX15" s="232"/>
+      <c r="AY15" s="233"/>
+      <c r="AZ15" s="233"/>
+      <c r="BA15" s="247">
+        <f t="shared" si="19"/>
+        <v>6.0496390791464145E-8</v>
+      </c>
+      <c r="BB15" s="234"/>
+      <c r="BC15" s="232"/>
+      <c r="BD15" s="233"/>
+      <c r="BE15" s="233"/>
+      <c r="BF15" s="247">
+        <f t="shared" si="20"/>
+        <v>2.1612895557484796E-4</v>
+      </c>
+      <c r="BG15" s="234"/>
+    </row>
+    <row r="16" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="43" t="s">
         <v>881</v>
       </c>
@@ -10773,18 +12428,18 @@
       </c>
       <c r="F16" s="43"/>
       <c r="G16" s="42">
-        <f t="shared" si="11"/>
+        <f t="shared" si="31"/>
         <v>1.3862943611198905E-4</v>
       </c>
       <c r="H16" s="43"/>
-      <c r="I16" s="42">
+      <c r="I16" s="223">
         <v>1.0035610685949183E-5</v>
       </c>
       <c r="J16" s="42">
-        <f>B23*R16^C23*(D23*S16^E23+F23*U16^G23)</f>
+        <f t="shared" si="21"/>
         <v>3.0587714365284148E-5</v>
       </c>
-      <c r="K16" s="42">
+      <c r="K16" s="223">
         <v>1.2989411467643282E-4</v>
       </c>
       <c r="L16" s="43" t="s">
@@ -10800,7 +12455,7 @@
         <v>838</v>
       </c>
       <c r="R16" s="4">
-        <f t="shared" si="10"/>
+        <f t="shared" si="30"/>
         <v>60</v>
       </c>
       <c r="S16" s="4">
@@ -10814,8 +12469,68 @@
         <f>'Drop-down lists'!S10</f>
         <v>482000</v>
       </c>
-    </row>
-    <row r="17" spans="1:21" s="11" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="V16" s="5"/>
+      <c r="W16" s="5">
+        <v>3.1300000000000001E-7</v>
+      </c>
+      <c r="X16" s="245">
+        <v>1.1800000000000001E-3</v>
+      </c>
+      <c r="Y16" s="232"/>
+      <c r="Z16" s="233"/>
+      <c r="AA16" s="233"/>
+      <c r="AB16" s="247">
+        <f t="shared" si="15"/>
+        <v>3.0587714365284148E-5</v>
+      </c>
+      <c r="AC16" s="245"/>
+      <c r="AD16" s="232"/>
+      <c r="AE16" s="233"/>
+      <c r="AF16" s="233"/>
+      <c r="AG16" s="247">
+        <f t="shared" si="16"/>
+        <v>3.0400351123367466E-5</v>
+      </c>
+      <c r="AH16" s="234"/>
+      <c r="AI16" s="232"/>
+      <c r="AJ16" s="233"/>
+      <c r="AK16" s="233"/>
+      <c r="AL16" s="233"/>
+      <c r="AM16" s="234"/>
+      <c r="AN16" s="232"/>
+      <c r="AO16" s="233"/>
+      <c r="AP16" s="233"/>
+      <c r="AQ16" s="247">
+        <f t="shared" si="17"/>
+        <v>6.5932977549445151E-5</v>
+      </c>
+      <c r="AR16" s="234"/>
+      <c r="AS16" s="232"/>
+      <c r="AT16" s="233"/>
+      <c r="AU16" s="233"/>
+      <c r="AV16" s="247">
+        <f t="shared" si="18"/>
+        <v>8.0391222994714338E-5</v>
+      </c>
+      <c r="AW16" s="234"/>
+      <c r="AX16" s="232"/>
+      <c r="AY16" s="233"/>
+      <c r="AZ16" s="233"/>
+      <c r="BA16" s="247">
+        <f t="shared" si="19"/>
+        <v>3.1339626641429535E-7</v>
+      </c>
+      <c r="BB16" s="234"/>
+      <c r="BC16" s="232"/>
+      <c r="BD16" s="233"/>
+      <c r="BE16" s="233"/>
+      <c r="BF16" s="247">
+        <f t="shared" si="20"/>
+        <v>2.635310038197716E-4</v>
+      </c>
+      <c r="BG16" s="234"/>
+    </row>
+    <row r="17" spans="1:59" s="11" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="60" t="s">
         <v>883</v>
       </c>
@@ -10837,14 +12552,14 @@
         <v>1.201860540707184E-5</v>
       </c>
       <c r="H17" s="60"/>
-      <c r="I17" s="44">
+      <c r="I17" s="224">
         <v>2.1351766919693532E-4</v>
       </c>
-      <c r="J17" s="44">
-        <f>B23*R17^C23*(D23*S17^E23+F23*U17^G23)</f>
+      <c r="J17" s="42">
+        <f t="shared" si="21"/>
         <v>5.0867301839797277E-4</v>
       </c>
-      <c r="K17" s="44">
+      <c r="K17" s="224">
         <v>3.1033329639430425E-3</v>
       </c>
       <c r="L17" s="60" t="s">
@@ -10878,8 +12593,45 @@
       <c r="U17" s="11">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:21" s="11" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W17" s="250"/>
+      <c r="X17" s="252"/>
+      <c r="Y17" s="232"/>
+      <c r="Z17" s="233"/>
+      <c r="AA17" s="233"/>
+      <c r="AB17" s="233"/>
+      <c r="AC17" s="245"/>
+      <c r="AD17" s="250"/>
+      <c r="AE17" s="251"/>
+      <c r="AF17" s="251"/>
+      <c r="AG17" s="251"/>
+      <c r="AH17" s="252"/>
+      <c r="AI17" s="250"/>
+      <c r="AJ17" s="251"/>
+      <c r="AK17" s="251"/>
+      <c r="AL17" s="251"/>
+      <c r="AM17" s="252"/>
+      <c r="AN17" s="250"/>
+      <c r="AO17" s="251"/>
+      <c r="AP17" s="251"/>
+      <c r="AQ17" s="251"/>
+      <c r="AR17" s="252"/>
+      <c r="AS17" s="250"/>
+      <c r="AT17" s="251"/>
+      <c r="AU17" s="251"/>
+      <c r="AV17" s="251"/>
+      <c r="AW17" s="252"/>
+      <c r="AX17" s="250"/>
+      <c r="AY17" s="251"/>
+      <c r="AZ17" s="251"/>
+      <c r="BA17" s="251"/>
+      <c r="BB17" s="252"/>
+      <c r="BC17" s="250"/>
+      <c r="BD17" s="251"/>
+      <c r="BE17" s="251"/>
+      <c r="BF17" s="251"/>
+      <c r="BG17" s="252"/>
+    </row>
+    <row r="18" spans="1:59" s="11" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="60" t="s">
         <v>884</v>
       </c>
@@ -10901,14 +12653,14 @@
         <v>7.9465494618955479E-5</v>
       </c>
       <c r="H18" s="60"/>
-      <c r="I18" s="44">
+      <c r="I18" s="224">
         <v>3.9120192104101118E-5</v>
       </c>
-      <c r="J18" s="44">
-        <f>B24*R18^C24*(D24*S18^E24+F24*U18^G24)</f>
+      <c r="J18" s="42">
+        <f>C$43*R18^D$43*(E$43*S18^F$43+G$43*U18^H$43)</f>
         <v>3.9120338116178696E-5</v>
       </c>
-      <c r="K18" s="44">
+      <c r="K18" s="224">
         <v>3.9120482637800647E-5</v>
       </c>
       <c r="L18" s="60" t="s">
@@ -10942,16 +12694,53 @@
       <c r="U18" s="11">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:21" s="11" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W18" s="253"/>
+      <c r="X18" s="255"/>
+      <c r="Y18" s="235"/>
+      <c r="Z18" s="236"/>
+      <c r="AA18" s="236"/>
+      <c r="AB18" s="236"/>
+      <c r="AC18" s="249"/>
+      <c r="AD18" s="253"/>
+      <c r="AE18" s="254"/>
+      <c r="AF18" s="254"/>
+      <c r="AG18" s="254"/>
+      <c r="AH18" s="255"/>
+      <c r="AI18" s="253"/>
+      <c r="AJ18" s="254"/>
+      <c r="AK18" s="254"/>
+      <c r="AL18" s="254"/>
+      <c r="AM18" s="255"/>
+      <c r="AN18" s="253"/>
+      <c r="AO18" s="254"/>
+      <c r="AP18" s="254"/>
+      <c r="AQ18" s="254"/>
+      <c r="AR18" s="255"/>
+      <c r="AS18" s="253"/>
+      <c r="AT18" s="254"/>
+      <c r="AU18" s="254"/>
+      <c r="AV18" s="254"/>
+      <c r="AW18" s="255"/>
+      <c r="AX18" s="253"/>
+      <c r="AY18" s="254"/>
+      <c r="AZ18" s="254"/>
+      <c r="BA18" s="254"/>
+      <c r="BB18" s="255"/>
+      <c r="BC18" s="253"/>
+      <c r="BD18" s="254"/>
+      <c r="BE18" s="254"/>
+      <c r="BF18" s="254"/>
+      <c r="BG18" s="255"/>
+    </row>
+    <row r="19" spans="1:59" s="11" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="181" t="s">
         <v>1014</v>
       </c>
     </row>
-    <row r="20" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="N20" s="11"/>
     </row>
-    <row r="21" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>232</v>
       </c>
@@ -10977,7 +12766,7 @@
       <c r="I21" s="3"/>
       <c r="J21" s="58"/>
     </row>
-    <row r="22" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
         <v>772</v>
       </c>
@@ -11009,7 +12798,7 @@
       <c r="I22" s="3"/>
       <c r="J22" s="58"/>
     </row>
-    <row r="23" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
         <v>235</v>
       </c>
@@ -11041,7 +12830,7 @@
       <c r="I23" s="5"/>
       <c r="J23" s="58"/>
     </row>
-    <row r="24" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>646</v>
       </c>
@@ -11073,13 +12862,676 @@
       <c r="I24" s="3"/>
       <c r="J24" s="58"/>
     </row>
-    <row r="25" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="J25" s="58"/>
+    </row>
+    <row r="26" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="4" t="str" cm="1">
+        <f t="array" ref="A26:H50">'Drop-down lists'!A2:H26</f>
+        <v>Polymer-specific empirical constants – Fragmentation</v>
+      </c>
+      <c r="B26" s="4">
+        <v>0</v>
+      </c>
+      <c r="C26" s="4">
+        <v>0</v>
+      </c>
+      <c r="D26" s="4">
+        <v>0</v>
+      </c>
+      <c r="E26" s="4">
+        <v>0</v>
+      </c>
+      <c r="F26" s="4">
+        <v>0</v>
+      </c>
+      <c r="G26" s="4">
+        <v>0</v>
+      </c>
+      <c r="H26" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="4" t="str">
+        <v>Index (i)</v>
+      </c>
+      <c r="B27" s="4" t="str">
+        <v>Polymer</v>
+      </c>
+      <c r="C27" s="4" t="str">
+        <v>a_i</v>
+      </c>
+      <c r="D27" s="4" t="str">
+        <v>delta_i</v>
+      </c>
+      <c r="E27" s="4" t="str">
+        <v>b_i</v>
+      </c>
+      <c r="F27" s="4" t="str">
+        <v>alpha_i</v>
+      </c>
+      <c r="G27" s="4" t="str">
+        <v>c_i</v>
+      </c>
+      <c r="H27" s="4" t="str">
+        <v>beta_i</v>
+      </c>
+    </row>
+    <row r="28" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="4">
+        <v>1</v>
+      </c>
+      <c r="B28" s="4" t="str">
+        <v>HDPE</v>
+      </c>
+      <c r="C28" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="D28" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E28" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F28" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G28" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H28" s="4" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="29" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="4">
+        <v>2</v>
+      </c>
+      <c r="B29" s="4" t="str">
+        <v>LDPE</v>
+      </c>
+      <c r="C29" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="D29" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E29" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F29" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G29" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H29" s="4" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="30" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="4">
+        <v>3</v>
+      </c>
+      <c r="B30" s="4" t="str">
+        <v>PE</v>
+      </c>
+      <c r="C30" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="D30" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E30" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F30" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G30" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H30" s="4" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="31" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="4">
+        <v>4</v>
+      </c>
+      <c r="B31" s="4" t="str">
+        <v>PP</v>
+      </c>
+      <c r="C31" s="4">
+        <v>4.6565907501850404E-6</v>
+      </c>
+      <c r="D31" s="4">
+        <v>2.2591669322139198</v>
+      </c>
+      <c r="E31" s="4">
+        <v>5.3412730896969978E-4</v>
+      </c>
+      <c r="F31" s="4">
+        <v>4.9999999999999827E-13</v>
+      </c>
+      <c r="G31" s="4">
+        <v>8.6756319826511703</v>
+      </c>
+      <c r="H31" s="4">
+        <v>1.4363331500021483</v>
+      </c>
+    </row>
+    <row r="32" spans="1:59" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="4">
+        <v>5</v>
+      </c>
+      <c r="B32" s="4" t="str">
+        <v>PS</v>
+      </c>
+      <c r="C32" s="4">
+        <v>7.2296289068305691E-3</v>
+      </c>
+      <c r="D32" s="4">
+        <v>3.9038558090829327</v>
+      </c>
+      <c r="E32" s="4">
+        <v>3.2687796728633455E-10</v>
+      </c>
+      <c r="F32" s="4">
+        <v>0.5497565488813938</v>
+      </c>
+      <c r="G32" s="4">
+        <v>55.746382030426993</v>
+      </c>
+      <c r="H32" s="4">
+        <v>4.9468547671349521</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="4">
+        <v>6</v>
+      </c>
+      <c r="B33" s="4" t="str">
+        <v>PET</v>
+      </c>
+      <c r="C33" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="D33" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E33" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F33" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G33" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H33" s="4" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="4">
+        <v>7</v>
+      </c>
+      <c r="B34" s="4" t="str">
+        <v>EPS</v>
+      </c>
+      <c r="C34" s="4">
+        <v>2.901642600553464E-2</v>
+      </c>
+      <c r="D34" s="4">
+        <v>9.3039280372760433E-12</v>
+      </c>
+      <c r="E34" s="4">
+        <v>1.6976290256311595E-7</v>
+      </c>
+      <c r="F34" s="4">
+        <v>4.9417608236281305</v>
+      </c>
+      <c r="G34" s="4">
+        <v>19.912251463764076</v>
+      </c>
+      <c r="H34" s="4">
+        <v>1.3446292576895287</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="4">
+        <v>8</v>
+      </c>
+      <c r="B35" s="4" t="str">
+        <v>PVC</v>
+      </c>
+      <c r="C35" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="D35" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E35" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F35" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G35" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H35" s="4" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="4">
+        <v>9</v>
+      </c>
+      <c r="B36" s="4" t="str">
+        <v>PLA</v>
+      </c>
+      <c r="C36" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="D36" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E36" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F36" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G36" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H36" s="4" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="4">
+        <v>10</v>
+      </c>
+      <c r="B37" s="4" t="str">
+        <v>PA</v>
+      </c>
+      <c r="C37" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="D37" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E37" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F37" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G37" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H37" s="4" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="4">
+        <v>0</v>
+      </c>
+      <c r="B38" s="4">
+        <v>0</v>
+      </c>
+      <c r="C38" s="4">
+        <v>0</v>
+      </c>
+      <c r="D38" s="4">
+        <v>0</v>
+      </c>
+      <c r="E38" s="4">
+        <v>0</v>
+      </c>
+      <c r="F38" s="4">
+        <v>0</v>
+      </c>
+      <c r="G38" s="4">
+        <v>0</v>
+      </c>
+      <c r="H38" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="4" t="str">
+        <v>Polymer-specific empirical constants – Degradation</v>
+      </c>
+      <c r="B39" s="4">
+        <v>0</v>
+      </c>
+      <c r="C39" s="4">
+        <v>0</v>
+      </c>
+      <c r="D39" s="4">
+        <v>0</v>
+      </c>
+      <c r="E39" s="4">
+        <v>0</v>
+      </c>
+      <c r="F39" s="4">
+        <v>0</v>
+      </c>
+      <c r="G39" s="4">
+        <v>0</v>
+      </c>
+      <c r="H39" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="4" t="str">
+        <v>Index (i)</v>
+      </c>
+      <c r="B40" s="4" t="str">
+        <v>Polymer</v>
+      </c>
+      <c r="C40" s="4" t="str">
+        <v>x_i</v>
+      </c>
+      <c r="D40" s="4" t="str">
+        <v>tau_i</v>
+      </c>
+      <c r="E40" s="4" t="str">
+        <v>y_i</v>
+      </c>
+      <c r="F40" s="4" t="str">
+        <v>theta_i</v>
+      </c>
+      <c r="G40" s="4" t="str">
+        <v>z_i</v>
+      </c>
+      <c r="H40" s="4" t="str">
+        <v>eta_i</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="4">
+        <v>1</v>
+      </c>
+      <c r="B41" s="4" t="str">
+        <v>HDPE</v>
+      </c>
+      <c r="C41" s="4">
+        <v>1.0262753023911369E-2</v>
+      </c>
+      <c r="D41" s="4">
+        <v>3.358408094206361E-11</v>
+      </c>
+      <c r="E41" s="4">
+        <v>2.1825283888841857E-3</v>
+      </c>
+      <c r="F41" s="4">
+        <v>0.29904863199407866</v>
+      </c>
+      <c r="G41" s="4">
+        <v>3.780320604053785E-4</v>
+      </c>
+      <c r="H41" s="4">
+        <v>0.21648776963088343</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="4">
+        <v>2</v>
+      </c>
+      <c r="B42" s="4" t="str">
+        <v>LDPE</v>
+      </c>
+      <c r="C42" s="4">
+        <v>1.1050589923981958E-2</v>
+      </c>
+      <c r="D42" s="4">
+        <v>4.9999999999999827E-13</v>
+      </c>
+      <c r="E42" s="4">
+        <v>1.0314560124374485E-2</v>
+      </c>
+      <c r="F42" s="4">
+        <v>4.362022267738264E-3</v>
+      </c>
+      <c r="G42" s="4">
+        <v>1.0475542749963076E-4</v>
+      </c>
+      <c r="H42" s="4">
+        <v>0.32405972126395782</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="4">
+        <v>3</v>
+      </c>
+      <c r="B43" s="4" t="str">
+        <v>PE</v>
+      </c>
+      <c r="C43" s="4">
+        <v>4.7218302973121193E-9</v>
+      </c>
+      <c r="D43" s="4">
+        <v>1.3476470812839827</v>
+      </c>
+      <c r="E43" s="4">
+        <v>3.6784226416775896E-4</v>
+      </c>
+      <c r="F43" s="4">
+        <v>4.9897636856199528</v>
+      </c>
+      <c r="G43" s="4">
+        <v>5.3315116606357247E-5</v>
+      </c>
+      <c r="H43" s="4">
+        <v>0.65085027677318608</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="4">
+        <v>4</v>
+      </c>
+      <c r="B44" s="4" t="str">
+        <v>PP</v>
+      </c>
+      <c r="C44" s="4">
+        <v>5.498191491131529E-3</v>
+      </c>
+      <c r="D44" s="4">
+        <v>1.3720790802151868E-2</v>
+      </c>
+      <c r="E44" s="4">
+        <v>1.7245229542043029E-2</v>
+      </c>
+      <c r="F44" s="4">
+        <v>0.70549281899550453</v>
+      </c>
+      <c r="G44" s="4">
+        <v>1.6158543822027385E-5</v>
+      </c>
+      <c r="H44" s="4">
+        <v>0.4421091864971286</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="4">
+        <v>5</v>
+      </c>
+      <c r="B45" s="4" t="str">
+        <v>PS</v>
+      </c>
+      <c r="C45" s="4">
+        <v>2.7325414959528186E-4</v>
+      </c>
+      <c r="D45" s="4">
+        <v>0.24329239036966804</v>
+      </c>
+      <c r="E45" s="4">
+        <v>1.4446952203994605E-2</v>
+      </c>
+      <c r="F45" s="4">
+        <v>1.0090731771779824</v>
+      </c>
+      <c r="G45" s="4">
+        <v>6.2330521521325821E-5</v>
+      </c>
+      <c r="H45" s="4">
+        <v>0.49603678909463539</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="4">
+        <v>6</v>
+      </c>
+      <c r="B46" s="4" t="str">
+        <v>PET</v>
+      </c>
+      <c r="C46" s="4">
+        <v>2.432762664179211E-4</v>
+      </c>
+      <c r="D46" s="4">
+        <v>0.79097577099168459</v>
+      </c>
+      <c r="E46" s="4">
+        <v>1.3261955767881682E-5</v>
+      </c>
+      <c r="F46" s="4">
+        <v>1.8763022076137708</v>
+      </c>
+      <c r="G46" s="4">
+        <v>1.5217890973559184E-2</v>
+      </c>
+      <c r="H46" s="4">
+        <v>7.8461949501476475E-2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="4">
+        <v>7</v>
+      </c>
+      <c r="B47" s="4" t="str">
+        <v>EPS</v>
+      </c>
+      <c r="C47" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="D47" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E47" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F47" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G47" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H47" s="4" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="4">
+        <v>8</v>
+      </c>
+      <c r="B48" s="4" t="str">
+        <v>PVC</v>
+      </c>
+      <c r="C48" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="D48" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E48" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F48" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G48" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H48" s="4" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="4">
+        <v>9</v>
+      </c>
+      <c r="B49" s="4" t="str">
+        <v>PLA</v>
+      </c>
+      <c r="C49" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="D49" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E49" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F49" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G49" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H49" s="4" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="4">
+        <v>10</v>
+      </c>
+      <c r="B50" s="4" t="str">
+        <v>PA</v>
+      </c>
+      <c r="C50" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="D50" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E50" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F50" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="G50" s="4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="H50" s="4" t="str">
+        <v>N/A</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="N2:P2"/>
   </mergeCells>
+  <conditionalFormatting sqref="AB14:AB16 Y12:AH13 AG14:AG16 AQ14:AQ16 AV14:AV16 BA14:BA16 Y11:BG11 AN12:BG13 BF14:BF16">
+    <cfRule type="top10" dxfId="6" priority="4" rank="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI12:AM12">
+    <cfRule type="top10" dxfId="5" priority="3" rank="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AR14:AU14 AW14:AZ14">
+    <cfRule type="top10" dxfId="2" priority="2" rank="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AR15:AU15 AW15:AZ15">
+    <cfRule type="top10" dxfId="1" priority="1" rank="1"/>
+  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation operator="greaterThan" showInputMessage="1" showErrorMessage="1" sqref="B21:C22 D22:G22" xr:uid="{8600E8B5-9C5C-2340-A471-9826A54D5F42}"/>
   </dataValidations>
@@ -13168,6 +15620,30 @@
     <sortCondition ref="A3:A36"/>
   </sortState>
   <mergeCells count="36">
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
@@ -13180,30 +15656,6 @@
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13766,29 +16218,29 @@
       </c>
     </row>
     <row r="2" spans="1:20" s="3" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="198" t="s">
+      <c r="A2" s="199" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="198"/>
-      <c r="C2" s="198"/>
-      <c r="D2" s="198"/>
-      <c r="E2" s="198"/>
-      <c r="F2" s="198"/>
-      <c r="G2" s="198"/>
-      <c r="H2" s="198"/>
-      <c r="J2" s="198" t="s">
+      <c r="B2" s="199"/>
+      <c r="C2" s="199"/>
+      <c r="D2" s="199"/>
+      <c r="E2" s="199"/>
+      <c r="F2" s="199"/>
+      <c r="G2" s="199"/>
+      <c r="H2" s="199"/>
+      <c r="J2" s="199" t="s">
         <v>226</v>
       </c>
-      <c r="K2" s="198"/>
-      <c r="L2" s="198"/>
-      <c r="M2" s="198"/>
-      <c r="O2" s="198" t="s">
+      <c r="K2" s="199"/>
+      <c r="L2" s="199"/>
+      <c r="M2" s="199"/>
+      <c r="O2" s="199" t="s">
         <v>763</v>
       </c>
-      <c r="P2" s="199"/>
-      <c r="Q2" s="199"/>
-      <c r="R2" s="199"/>
-      <c r="S2" s="199"/>
+      <c r="P2" s="200"/>
+      <c r="Q2" s="200"/>
+      <c r="R2" s="200"/>
+      <c r="S2" s="200"/>
     </row>
     <row r="3" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="39" t="s">
@@ -14253,13 +16705,13 @@
         <v>48</v>
       </c>
       <c r="N11" s="9"/>
-      <c r="O11" s="197" t="s">
+      <c r="O11" s="198" t="s">
         <v>810</v>
       </c>
-      <c r="P11" s="197"/>
-      <c r="Q11" s="197"/>
-      <c r="R11" s="197"/>
-      <c r="S11" s="197"/>
+      <c r="P11" s="198"/>
+      <c r="Q11" s="198"/>
+      <c r="R11" s="198"/>
+      <c r="S11" s="198"/>
     </row>
     <row r="12" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="27">
@@ -14293,11 +16745,11 @@
       <c r="K12" s="27"/>
       <c r="L12" s="27"/>
       <c r="M12" s="27"/>
-      <c r="O12" s="197"/>
-      <c r="P12" s="197"/>
-      <c r="Q12" s="197"/>
-      <c r="R12" s="197"/>
-      <c r="S12" s="197"/>
+      <c r="O12" s="198"/>
+      <c r="P12" s="198"/>
+      <c r="Q12" s="198"/>
+      <c r="R12" s="198"/>
+      <c r="S12" s="198"/>
     </row>
     <row r="13" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="27">
@@ -14331,11 +16783,11 @@
       <c r="K13" s="27"/>
       <c r="L13" s="27"/>
       <c r="M13" s="27"/>
-      <c r="O13" s="197"/>
-      <c r="P13" s="197"/>
-      <c r="Q13" s="197"/>
-      <c r="R13" s="197"/>
-      <c r="S13" s="197"/>
+      <c r="O13" s="198"/>
+      <c r="P13" s="198"/>
+      <c r="Q13" s="198"/>
+      <c r="R13" s="198"/>
+      <c r="S13" s="198"/>
       <c r="T13" s="3"/>
     </row>
     <row r="14" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -14353,16 +16805,16 @@
       <c r="M14" s="40"/>
     </row>
     <row r="15" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="198" t="s">
+      <c r="A15" s="199" t="s">
         <v>52</v>
       </c>
-      <c r="B15" s="198"/>
-      <c r="C15" s="198"/>
-      <c r="D15" s="198"/>
-      <c r="E15" s="198"/>
-      <c r="F15" s="198"/>
-      <c r="G15" s="198"/>
-      <c r="H15" s="198"/>
+      <c r="B15" s="199"/>
+      <c r="C15" s="199"/>
+      <c r="D15" s="199"/>
+      <c r="E15" s="199"/>
+      <c r="F15" s="199"/>
+      <c r="G15" s="199"/>
+      <c r="H15" s="199"/>
       <c r="O15" s="164" t="s">
         <v>731</v>
       </c>
@@ -14397,12 +16849,12 @@
         <v>17</v>
       </c>
       <c r="I16" s="3"/>
-      <c r="J16" s="198" t="s">
+      <c r="J16" s="199" t="s">
         <v>729</v>
       </c>
-      <c r="K16" s="198"/>
-      <c r="L16" s="198"/>
-      <c r="M16" s="198"/>
+      <c r="K16" s="199"/>
+      <c r="L16" s="199"/>
+      <c r="M16" s="199"/>
       <c r="O16" s="39" t="s">
         <v>738</v>
       </c>
@@ -14798,12 +17250,12 @@
         <v>705</v>
       </c>
       <c r="I24" s="7"/>
-      <c r="J24" s="198" t="s">
+      <c r="J24" s="199" t="s">
         <v>742</v>
       </c>
-      <c r="K24" s="198"/>
-      <c r="L24" s="198"/>
-      <c r="M24" s="198" t="s">
+      <c r="K24" s="199"/>
+      <c r="L24" s="199"/>
+      <c r="M24" s="199" t="s">
         <v>741</v>
       </c>
       <c r="O24" s="27" t="s">
@@ -14851,10 +17303,10 @@
       <c r="J25" s="17" t="s">
         <v>740</v>
       </c>
-      <c r="K25" s="195" t="s">
+      <c r="K25" s="197" t="s">
         <v>743</v>
       </c>
-      <c r="L25" s="195"/>
+      <c r="L25" s="197"/>
       <c r="M25" s="17" t="s">
         <v>744</v>
       </c>
@@ -14903,10 +17355,10 @@
       <c r="J26" s="27" t="s">
         <v>748</v>
       </c>
-      <c r="K26" s="200" t="s">
+      <c r="K26" s="196" t="s">
         <v>705</v>
       </c>
-      <c r="L26" s="200"/>
+      <c r="L26" s="196"/>
       <c r="M26" s="27" t="s">
         <v>705</v>
       </c>
@@ -14937,10 +17389,10 @@
       <c r="J27" s="40" t="s">
         <v>747</v>
       </c>
-      <c r="K27" s="196" t="s">
+      <c r="K27" s="195" t="s">
         <v>746</v>
       </c>
-      <c r="L27" s="196"/>
+      <c r="L27" s="195"/>
       <c r="M27" s="40">
         <v>5.0000000000000001E-3</v>
       </c>
@@ -14967,10 +17419,10 @@
       <c r="J28" s="40" t="s">
         <v>965</v>
       </c>
-      <c r="K28" s="196" t="s">
+      <c r="K28" s="195" t="s">
         <v>966</v>
       </c>
-      <c r="L28" s="196"/>
+      <c r="L28" s="195"/>
       <c r="M28" s="40">
         <v>0.02</v>
       </c>
@@ -15002,10 +17454,10 @@
       <c r="J29" s="40" t="s">
         <v>967</v>
       </c>
-      <c r="K29" s="196" t="s">
+      <c r="K29" s="195" t="s">
         <v>968</v>
       </c>
-      <c r="L29" s="196"/>
+      <c r="L29" s="195"/>
       <c r="M29" s="40">
         <v>0.2</v>
       </c>
@@ -15021,10 +17473,10 @@
       <c r="J30" s="40" t="s">
         <v>969</v>
       </c>
-      <c r="K30" s="196" t="s">
+      <c r="K30" s="195" t="s">
         <v>970</v>
       </c>
-      <c r="L30" s="196"/>
+      <c r="L30" s="195"/>
       <c r="M30" s="40">
         <v>0.5</v>
       </c>
@@ -15040,10 +17492,10 @@
       <c r="J31" s="27" t="s">
         <v>971</v>
       </c>
-      <c r="K31" s="196" t="s">
+      <c r="K31" s="195" t="s">
         <v>972</v>
       </c>
-      <c r="L31" s="196"/>
+      <c r="L31" s="195"/>
       <c r="M31" s="155">
         <v>1</v>
       </c>
@@ -15083,11 +17535,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="K26:L26"/>
     <mergeCell ref="K25:L25"/>
     <mergeCell ref="K27:L27"/>
     <mergeCell ref="O11:S13"/>
@@ -15097,6 +17544,11 @@
     <mergeCell ref="J24:M24"/>
     <mergeCell ref="O2:S2"/>
     <mergeCell ref="J16:M16"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="K26:L26"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <dataValidations count="1">
@@ -24079,7 +26531,7 @@
         <v>426</v>
       </c>
       <c r="D3" s="28">
-        <f t="shared" ref="D3:D28" si="0">-LN(1-J3/100)/I3</f>
+        <f>-LN(1-J3/100)/I3</f>
         <v>5.0226359178605949E-5</v>
       </c>
       <c r="E3" s="137">
@@ -24142,7 +26594,7 @@
         <v>426</v>
       </c>
       <c r="D4" s="28">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="D3:D28" si="0">-LN(1-J4/100)/I4</f>
         <v>2.2023185715519423E-8</v>
       </c>
       <c r="E4" s="137">
@@ -33265,7 +35717,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81E699B8-79ED-0D4F-9893-DEE59A5FDA00}">
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="15.83203125" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" style="151" customWidth="1"/>
@@ -34110,7 +36562,7 @@
         <v>628</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>611</v>
+        <v>7</v>
       </c>
       <c r="C39" s="5">
         <v>4.6565907501850404E-6</v>
@@ -34650,37 +37102,293 @@
       <c r="J62" s="6"/>
     </row>
     <row r="63" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C63" s="5"/>
-      <c r="D63" s="5"/>
-      <c r="E63" s="5"/>
+      <c r="A63" s="189" t="s">
+        <v>635</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>619</v>
+      </c>
+      <c r="C63" s="5">
+        <v>2.432762664179211E-4</v>
+      </c>
+      <c r="D63" s="5">
+        <v>2.9524825547148014E-4</v>
+      </c>
+      <c r="E63" s="6">
+        <v>2.9524826190579095E-2</v>
+      </c>
+      <c r="F63" s="189" t="s">
+        <v>640</v>
+      </c>
+      <c r="G63" s="1" t="s">
+        <v>611</v>
+      </c>
+      <c r="H63" s="5"/>
+      <c r="I63" s="5"/>
+      <c r="J63" s="6"/>
     </row>
     <row r="64" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C64" s="5"/>
-      <c r="D64" s="5"/>
-      <c r="E64" s="5"/>
-    </row>
-    <row r="65" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C65" s="5"/>
-      <c r="D65" s="5"/>
-      <c r="E65" s="5"/>
-    </row>
-    <row r="66" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C66" s="5"/>
-      <c r="D66" s="5"/>
-      <c r="E66" s="5"/>
-    </row>
-    <row r="67" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C67" s="5"/>
-      <c r="D67" s="5"/>
-      <c r="E67" s="5"/>
-    </row>
-    <row r="68" spans="3:5" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C68" s="5"/>
-      <c r="D68" s="5"/>
-      <c r="E68" s="5"/>
+      <c r="A64" s="189"/>
+      <c r="B64" s="1" t="s">
+        <v>620</v>
+      </c>
+      <c r="C64" s="5">
+        <v>0.79097577099168459</v>
+      </c>
+      <c r="D64" s="5">
+        <v>0.19332889713928206</v>
+      </c>
+      <c r="E64" s="6">
+        <v>19.514951094930019</v>
+      </c>
+      <c r="F64" s="189"/>
+      <c r="G64" s="1" t="s">
+        <v>612</v>
+      </c>
+      <c r="H64" s="5"/>
+      <c r="I64" s="5"/>
+      <c r="J64" s="6"/>
+    </row>
+    <row r="65" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="189"/>
+      <c r="B65" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C65" s="5">
+        <v>1.3261955767881682E-5</v>
+      </c>
+      <c r="D65" s="5">
+        <v>2.1960388534196288E-5</v>
+      </c>
+      <c r="E65" s="167">
+        <v>2.1960388536843931E-3</v>
+      </c>
+      <c r="F65" s="189"/>
+      <c r="G65" s="1" t="s">
+        <v>613</v>
+      </c>
+      <c r="H65" s="5"/>
+      <c r="I65" s="5"/>
+      <c r="J65" s="6"/>
+    </row>
+    <row r="66" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="189"/>
+      <c r="B66" s="1" t="s">
+        <v>621</v>
+      </c>
+      <c r="C66" s="5">
+        <v>1.8763022076137708</v>
+      </c>
+      <c r="D66" s="5">
+        <v>0.22318783126059411</v>
+      </c>
+      <c r="E66" s="6">
+        <v>22.599629483353922</v>
+      </c>
+      <c r="F66" s="189"/>
+      <c r="G66" s="1" t="s">
+        <v>614</v>
+      </c>
+      <c r="H66" s="5"/>
+      <c r="I66" s="5"/>
+      <c r="J66" s="6"/>
+    </row>
+    <row r="67" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A67" s="189"/>
+      <c r="B67" s="1" t="s">
+        <v>622</v>
+      </c>
+      <c r="C67" s="5">
+        <v>1.5217890973559184E-2</v>
+      </c>
+      <c r="D67" s="5">
+        <v>4.4013893320794464E-6</v>
+      </c>
+      <c r="E67" s="173">
+        <v>4.4013893321007629E-4</v>
+      </c>
+      <c r="F67" s="189"/>
+      <c r="G67" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="H67" s="5"/>
+      <c r="I67" s="5"/>
+      <c r="J67" s="6"/>
+    </row>
+    <row r="68" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="189"/>
+      <c r="B68" s="1" t="s">
+        <v>623</v>
+      </c>
+      <c r="C68" s="5">
+        <v>7.8461949501476475E-2</v>
+      </c>
+      <c r="D68" s="5">
+        <v>4.5684842445671371E-2</v>
+      </c>
+      <c r="E68" s="6">
+        <v>4.5708690077504608</v>
+      </c>
+      <c r="F68" s="189"/>
+      <c r="G68" s="1" t="s">
+        <v>615</v>
+      </c>
+      <c r="H68" s="5"/>
+      <c r="I68" s="5"/>
+      <c r="J68" s="6"/>
+    </row>
+    <row r="69" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="189" t="s">
+        <v>632</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>611</v>
+      </c>
+      <c r="C69" s="5">
+        <v>2.901642600553464E-2</v>
+      </c>
+      <c r="D69" s="5">
+        <v>4.1834802275052388E-2</v>
+      </c>
+      <c r="E69" s="6">
+        <v>4.1853113252749736</v>
+      </c>
+      <c r="F69" s="189" t="s">
+        <v>641</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>619</v>
+      </c>
+      <c r="H69" s="5"/>
+      <c r="I69" s="5"/>
+      <c r="J69" s="6"/>
+    </row>
+    <row r="70" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="189"/>
+      <c r="B70" s="1" t="s">
+        <v>612</v>
+      </c>
+      <c r="C70" s="5">
+        <v>9.3039280372760433E-12</v>
+      </c>
+      <c r="D70" s="5">
+        <v>0.54476707002904701</v>
+      </c>
+      <c r="E70" s="6">
+        <v>58.779874030329701</v>
+      </c>
+      <c r="F70" s="189"/>
+      <c r="G70" s="1" t="s">
+        <v>620</v>
+      </c>
+      <c r="H70" s="5"/>
+      <c r="I70" s="5"/>
+      <c r="J70" s="6"/>
+    </row>
+    <row r="71" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="189"/>
+      <c r="B71" s="1" t="s">
+        <v>613</v>
+      </c>
+      <c r="C71" s="5">
+        <v>1.6976290256311595E-7</v>
+      </c>
+      <c r="D71" s="5">
+        <v>8.8342055745412053E-7</v>
+      </c>
+      <c r="E71" s="173">
+        <v>8.8342055745429285E-5</v>
+      </c>
+      <c r="F71" s="189"/>
+      <c r="G71" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="H71" s="5"/>
+      <c r="I71" s="5"/>
+      <c r="J71" s="6"/>
+    </row>
+    <row r="72" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="189"/>
+      <c r="B72" s="1" t="s">
+        <v>614</v>
+      </c>
+      <c r="C72" s="5">
+        <v>4.9417608236281305</v>
+      </c>
+      <c r="D72" s="5">
+        <v>2.2258288818141088</v>
+      </c>
+      <c r="E72" s="6">
+        <v>1186.5299752448714</v>
+      </c>
+      <c r="F72" s="189"/>
+      <c r="G72" s="1" t="s">
+        <v>621</v>
+      </c>
+      <c r="H72" s="5"/>
+      <c r="I72" s="5"/>
+      <c r="J72" s="6"/>
+    </row>
+    <row r="73" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A73" s="189"/>
+      <c r="B73" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C73" s="5">
+        <v>19.912251463764076</v>
+      </c>
+      <c r="D73" s="5">
+        <v>1.3385794980254835E-4</v>
+      </c>
+      <c r="E73" s="6">
+        <v>1.3385795040216341E-2</v>
+      </c>
+      <c r="F73" s="189"/>
+      <c r="G73" s="1" t="s">
+        <v>622</v>
+      </c>
+      <c r="H73" s="5"/>
+      <c r="I73" s="5"/>
+      <c r="J73" s="6"/>
+    </row>
+    <row r="74" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A74" s="189"/>
+      <c r="B74" s="1" t="s">
+        <v>615</v>
+      </c>
+      <c r="C74" s="5">
+        <v>1.3446292576895287</v>
+      </c>
+      <c r="D74" s="5">
+        <v>0.26892862004663609</v>
+      </c>
+      <c r="E74" s="6">
+        <v>27.38650884744699</v>
+      </c>
+      <c r="F74" s="189"/>
+      <c r="G74" s="1" t="s">
+        <v>623</v>
+      </c>
+      <c r="H74" s="5"/>
+      <c r="I74" s="5"/>
+      <c r="J74" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="24">
+    <mergeCell ref="A63:A68"/>
+    <mergeCell ref="A69:A74"/>
+    <mergeCell ref="F63:F68"/>
+    <mergeCell ref="F69:F74"/>
+    <mergeCell ref="F45:F50"/>
+    <mergeCell ref="F51:F56"/>
+    <mergeCell ref="F57:F62"/>
+    <mergeCell ref="A33:A38"/>
+    <mergeCell ref="A39:A44"/>
+    <mergeCell ref="A45:A50"/>
+    <mergeCell ref="A51:A56"/>
+    <mergeCell ref="A57:A62"/>
+    <mergeCell ref="F33:F38"/>
+    <mergeCell ref="F39:F44"/>
     <mergeCell ref="F3:F8"/>
     <mergeCell ref="F9:F14"/>
     <mergeCell ref="A15:A20"/>
@@ -34691,16 +37399,6 @@
     <mergeCell ref="F27:F32"/>
     <mergeCell ref="A3:A8"/>
     <mergeCell ref="A9:A14"/>
-    <mergeCell ref="F45:F50"/>
-    <mergeCell ref="F51:F56"/>
-    <mergeCell ref="F57:F62"/>
-    <mergeCell ref="A33:A38"/>
-    <mergeCell ref="A39:A44"/>
-    <mergeCell ref="A45:A50"/>
-    <mergeCell ref="A51:A56"/>
-    <mergeCell ref="A57:A62"/>
-    <mergeCell ref="F33:F38"/>
-    <mergeCell ref="F39:F44"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -38598,33 +41296,33 @@
       <c r="R1" s="162"/>
     </row>
     <row r="2" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="215" t="s">
+      <c r="A2" s="216" t="s">
         <v>668</v>
       </c>
-      <c r="B2" s="215"/>
-      <c r="C2" s="215"/>
-      <c r="D2" s="215"/>
-      <c r="E2" s="215"/>
-      <c r="F2" s="216" t="s">
+      <c r="B2" s="216"/>
+      <c r="C2" s="216"/>
+      <c r="D2" s="216"/>
+      <c r="E2" s="216"/>
+      <c r="F2" s="217" t="s">
         <v>669</v>
       </c>
-      <c r="G2" s="216"/>
-      <c r="H2" s="216"/>
-      <c r="I2" s="216"/>
-      <c r="J2" s="216"/>
-      <c r="K2" s="218" t="s">
+      <c r="G2" s="217"/>
+      <c r="H2" s="217"/>
+      <c r="I2" s="217"/>
+      <c r="J2" s="217"/>
+      <c r="K2" s="219" t="s">
         <v>983</v>
       </c>
-      <c r="L2" s="218"/>
-      <c r="M2" s="218"/>
-      <c r="N2" s="218"/>
-      <c r="O2" s="218"/>
-      <c r="P2" s="218"/>
-      <c r="Q2" s="218"/>
-      <c r="R2" s="218"/>
-      <c r="S2" s="218"/>
-      <c r="T2" s="218"/>
-      <c r="U2" s="218"/>
+      <c r="L2" s="219"/>
+      <c r="M2" s="219"/>
+      <c r="N2" s="219"/>
+      <c r="O2" s="219"/>
+      <c r="P2" s="219"/>
+      <c r="Q2" s="219"/>
+      <c r="R2" s="219"/>
+      <c r="S2" s="219"/>
+      <c r="T2" s="219"/>
+      <c r="U2" s="219"/>
     </row>
     <row r="3" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="50" t="s">
@@ -38767,7 +41465,7 @@
         <f t="shared" ref="T4:T45" si="1">MAX(L4:Q4)</f>
         <v>1.2137301257607254</v>
       </c>
-      <c r="U4" s="219">
+      <c r="U4" s="220">
         <v>2</v>
       </c>
     </row>
@@ -38847,7 +41545,7 @@
         <f t="shared" si="1"/>
         <v>3.6973644778946788</v>
       </c>
-      <c r="U5" s="219"/>
+      <c r="U5" s="220"/>
     </row>
     <row r="6" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="83" t="s">
@@ -38925,7 +41623,7 @@
         <f t="shared" si="1"/>
         <v>0.70238237366234268</v>
       </c>
-      <c r="U6" s="219"/>
+      <c r="U6" s="220"/>
     </row>
     <row r="7" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="83" t="s">
@@ -39003,7 +41701,7 @@
         <f t="shared" si="1"/>
         <v>0.99518612453060507</v>
       </c>
-      <c r="U7" s="219"/>
+      <c r="U7" s="220"/>
     </row>
     <row r="8" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="83" t="s">
@@ -39081,7 +41779,7 @@
         <f t="shared" si="1"/>
         <v>698.43657647937516</v>
       </c>
-      <c r="U8" s="219"/>
+      <c r="U8" s="220"/>
     </row>
     <row r="9" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="83" t="s">
@@ -39159,7 +41857,7 @@
         <f t="shared" si="1"/>
         <v>134.82257640520913</v>
       </c>
-      <c r="U9" s="219"/>
+      <c r="U9" s="220"/>
     </row>
     <row r="10" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="83" t="s">
@@ -39237,7 +41935,7 @@
         <f t="shared" si="1"/>
         <v>10.096983699271892</v>
       </c>
-      <c r="U10" s="219">
+      <c r="U10" s="220">
         <v>6</v>
       </c>
     </row>
@@ -39317,7 +42015,7 @@
         <f t="shared" si="1"/>
         <v>3.046282200153263</v>
       </c>
-      <c r="U11" s="219"/>
+      <c r="U11" s="220"/>
     </row>
     <row r="12" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="83" t="s">
@@ -39395,7 +42093,7 @@
         <f t="shared" si="1"/>
         <v>3.8074444162573093</v>
       </c>
-      <c r="U12" s="219"/>
+      <c r="U12" s="220"/>
     </row>
     <row r="13" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="83" t="s">
@@ -39473,7 +42171,7 @@
         <f t="shared" si="1"/>
         <v>8.4089134569927921</v>
       </c>
-      <c r="U13" s="219"/>
+      <c r="U13" s="220"/>
     </row>
     <row r="14" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="83" t="s">
@@ -39551,7 +42249,7 @@
         <f t="shared" si="1"/>
         <v>575.44635471713161</v>
       </c>
-      <c r="U14" s="219"/>
+      <c r="U14" s="220"/>
     </row>
     <row r="15" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="83" t="s">
@@ -39629,7 +42327,7 @@
         <f t="shared" si="1"/>
         <v>111.08118151117561</v>
       </c>
-      <c r="U15" s="219"/>
+      <c r="U15" s="220"/>
     </row>
     <row r="16" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="83" t="s">
@@ -39707,7 +42405,7 @@
         <f t="shared" si="1"/>
         <v>4.5497270531392493</v>
       </c>
-      <c r="U16" s="219">
+      <c r="U16" s="220">
         <v>4</v>
       </c>
     </row>
@@ -39787,7 +42485,7 @@
         <f t="shared" si="1"/>
         <v>0.87433736936969564</v>
       </c>
-      <c r="U17" s="219"/>
+      <c r="U17" s="220"/>
     </row>
     <row r="18" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="83" t="s">
@@ -39865,7 +42563,7 @@
         <f t="shared" si="1"/>
         <v>1.6275040385171768</v>
       </c>
-      <c r="U18" s="219"/>
+      <c r="U18" s="220"/>
     </row>
     <row r="19" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="83" t="s">
@@ -39943,7 +42641,7 @@
         <f t="shared" si="1"/>
         <v>3.5944163892089054</v>
       </c>
-      <c r="U19" s="219"/>
+      <c r="U19" s="220"/>
     </row>
     <row r="20" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="83" t="s">
@@ -40021,7 +42719,7 @@
         <f t="shared" si="1"/>
         <v>188.90119723254139</v>
       </c>
-      <c r="U20" s="219"/>
+      <c r="U20" s="220"/>
     </row>
     <row r="21" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="83" t="s">
@@ -40099,7 +42797,7 @@
         <f t="shared" si="1"/>
         <v>36.464507951885402</v>
       </c>
-      <c r="U21" s="219"/>
+      <c r="U21" s="220"/>
     </row>
     <row r="22" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="83" t="s">
@@ -40177,7 +42875,7 @@
         <f t="shared" si="1"/>
         <v>3.7778094298488849</v>
       </c>
-      <c r="U22" s="219">
+      <c r="U22" s="220">
         <v>5</v>
       </c>
     </row>
@@ -40257,7 +42955,7 @@
         <f t="shared" si="1"/>
         <v>3.7704716371132965</v>
       </c>
-      <c r="U23" s="219"/>
+      <c r="U23" s="220"/>
     </row>
     <row r="24" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="83" t="s">
@@ -40335,7 +43033,7 @@
         <f t="shared" si="1"/>
         <v>11.485920634320969</v>
       </c>
-      <c r="U24" s="219"/>
+      <c r="U24" s="220"/>
     </row>
     <row r="25" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
@@ -40402,7 +43100,7 @@
         <f t="shared" si="1"/>
         <v>3.091561275896912</v>
       </c>
-      <c r="U25" s="219"/>
+      <c r="U25" s="220"/>
     </row>
     <row r="26" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
@@ -40469,7 +43167,7 @@
         <f t="shared" si="1"/>
         <v>2169.7041591411821</v>
       </c>
-      <c r="U26" s="219"/>
+      <c r="U26" s="220"/>
     </row>
     <row r="27" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
@@ -40536,7 +43234,7 @@
         <f t="shared" si="1"/>
         <v>418.82844430492156</v>
       </c>
-      <c r="U27" s="219"/>
+      <c r="U27" s="220"/>
     </row>
     <row r="28" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C28" s="5"/>
@@ -40597,7 +43295,7 @@
         <f t="shared" si="1"/>
         <v>2.6834498872986985</v>
       </c>
-      <c r="U28" s="219">
+      <c r="U28" s="220">
         <v>3</v>
       </c>
     </row>
@@ -40659,7 +43357,7 @@
         <f t="shared" si="1"/>
         <v>1.2196011337408867</v>
       </c>
-      <c r="U29" s="219"/>
+      <c r="U29" s="220"/>
     </row>
     <row r="30" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F30" s="34" t="s">
@@ -40719,7 +43417,7 @@
         <f t="shared" si="1"/>
         <v>3.7152492250016027</v>
       </c>
-      <c r="U30" s="219"/>
+      <c r="U30" s="220"/>
     </row>
     <row r="31" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F31" s="34" t="s">
@@ -40779,7 +43477,7 @@
         <f t="shared" si="1"/>
         <v>0.73385398939109214</v>
       </c>
-      <c r="U31" s="219"/>
+      <c r="U31" s="220"/>
     </row>
     <row r="32" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F32" s="34" t="s">
@@ -40839,7 +43537,7 @@
         <f t="shared" si="1"/>
         <v>701.81502662007426</v>
       </c>
-      <c r="U32" s="219"/>
+      <c r="U32" s="220"/>
     </row>
     <row r="33" spans="6:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F33" s="34" t="s">
@@ -40899,7 +43597,7 @@
         <f t="shared" si="1"/>
         <v>135.474734908307</v>
       </c>
-      <c r="U33" s="219"/>
+      <c r="U33" s="220"/>
     </row>
     <row r="34" spans="6:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F34" s="34" t="s">
@@ -40959,7 +43657,7 @@
         <f t="shared" si="1"/>
         <v>2.2612063527306732</v>
       </c>
-      <c r="U34" s="219">
+      <c r="U34" s="220">
         <v>0</v>
       </c>
     </row>
@@ -41021,7 +43719,7 @@
         <f t="shared" si="1"/>
         <v>0.46480643421499973</v>
       </c>
-      <c r="U35" s="219"/>
+      <c r="U35" s="220"/>
     </row>
     <row r="36" spans="6:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F36" s="34" t="s">
@@ -41081,7 +43779,7 @@
         <f t="shared" si="1"/>
         <v>0.53160993742046714</v>
       </c>
-      <c r="U36" s="219"/>
+      <c r="U36" s="220"/>
     </row>
     <row r="37" spans="6:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F37" s="34" t="s">
@@ -41141,7 +43839,7 @@
         <f t="shared" si="1"/>
         <v>0.61816649231153897</v>
       </c>
-      <c r="U37" s="219"/>
+      <c r="U37" s="220"/>
     </row>
     <row r="38" spans="6:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F38" s="34" t="s">
@@ -41201,7 +43899,7 @@
         <f t="shared" si="1"/>
         <v>0.84264899576974117</v>
       </c>
-      <c r="U38" s="219"/>
+      <c r="U38" s="220"/>
     </row>
     <row r="39" spans="6:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F39" s="34" t="s">
@@ -41261,7 +43959,7 @@
         <f t="shared" si="1"/>
         <v>0.82012724287521843</v>
       </c>
-      <c r="U39" s="219"/>
+      <c r="U39" s="220"/>
     </row>
     <row r="40" spans="6:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F40" s="34" t="s">
@@ -41321,7 +44019,7 @@
         <f t="shared" si="1"/>
         <v>2.7571408856061055</v>
       </c>
-      <c r="U40" s="219">
+      <c r="U40" s="220">
         <v>1</v>
       </c>
     </row>
@@ -41383,7 +44081,7 @@
         <f t="shared" si="1"/>
         <v>0.56674917002570491</v>
       </c>
-      <c r="U41" s="219"/>
+      <c r="U41" s="220"/>
     </row>
     <row r="42" spans="6:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F42" s="34" t="s">
@@ -41443,7 +44141,7 @@
         <f t="shared" si="1"/>
         <v>0.64820421713676823</v>
       </c>
-      <c r="U42" s="219"/>
+      <c r="U42" s="220"/>
     </row>
     <row r="43" spans="6:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F43" s="34" t="s">
@@ -41503,7 +44201,7 @@
         <f t="shared" si="1"/>
         <v>0.75374461424346617</v>
       </c>
-      <c r="U43" s="219"/>
+      <c r="U43" s="220"/>
     </row>
     <row r="44" spans="6:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F44" s="34" t="s">
@@ -41563,7 +44261,7 @@
         <f t="shared" si="1"/>
         <v>1.0274612910254823</v>
       </c>
-      <c r="U44" s="219"/>
+      <c r="U44" s="220"/>
     </row>
     <row r="45" spans="6:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F45" s="34" t="s">
@@ -41623,7 +44321,7 @@
         <f t="shared" si="1"/>
         <v>5.1804126215495589</v>
       </c>
-      <c r="U45" s="219"/>
+      <c r="U45" s="220"/>
     </row>
     <row r="46" spans="6:21" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F46" s="4" t="s">
@@ -41633,16 +44331,16 @@
         <f>GEOMEAN(H4:H10)</f>
         <v>2.0452304464973529E-4</v>
       </c>
-      <c r="K46" s="217" t="s">
+      <c r="K46" s="218" t="s">
         <v>984</v>
       </c>
-      <c r="L46" s="217"/>
-      <c r="M46" s="217"/>
-      <c r="N46" s="217"/>
-      <c r="O46" s="217"/>
-      <c r="P46" s="217"/>
-      <c r="Q46" s="217"/>
-      <c r="R46" s="217"/>
+      <c r="L46" s="218"/>
+      <c r="M46" s="218"/>
+      <c r="N46" s="218"/>
+      <c r="O46" s="218"/>
+      <c r="P46" s="218"/>
+      <c r="Q46" s="218"/>
+      <c r="R46" s="218"/>
       <c r="S46" s="8"/>
       <c r="T46" s="8"/>
     </row>
@@ -41716,7 +44414,7 @@
         <f>MAX(L48:N48)</f>
         <v>13.426460997516173</v>
       </c>
-      <c r="R48" s="220">
+      <c r="R48" s="215">
         <v>3</v>
       </c>
     </row>
@@ -41755,7 +44453,7 @@
         <f t="shared" ref="Q49:Q51" si="64">MAX(L49:N49)</f>
         <v>0.1381649642343851</v>
       </c>
-      <c r="R49" s="220"/>
+      <c r="R49" s="215"/>
     </row>
     <row r="50" spans="6:18" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F50" s="4" t="s">
@@ -41792,7 +44490,7 @@
         <f t="shared" si="64"/>
         <v>1.2760981964756606</v>
       </c>
-      <c r="R50" s="220"/>
+      <c r="R50" s="215"/>
     </row>
     <row r="51" spans="6:18" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F51" s="4" t="s">
@@ -41829,7 +44527,7 @@
         <f t="shared" si="64"/>
         <v>7.9699539295837248E+17</v>
       </c>
-      <c r="R51" s="220"/>
+      <c r="R51" s="215"/>
     </row>
     <row r="52" spans="6:18" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="K52" s="157" t="s">
@@ -41859,7 +44557,7 @@
         <f t="shared" ref="Q52:Q55" si="70">MAX(L52:N52)</f>
         <v>0.28554693625373867</v>
       </c>
-      <c r="R52" s="220">
+      <c r="R52" s="215">
         <v>1</v>
       </c>
     </row>
@@ -41891,7 +44589,7 @@
         <f t="shared" si="70"/>
         <v>2.2325593132868631E-2</v>
       </c>
-      <c r="R53" s="220"/>
+      <c r="R53" s="215"/>
     </row>
     <row r="54" spans="6:18" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="K54" s="157" t="s">
@@ -41921,7 +44619,7 @@
         <f t="shared" si="70"/>
         <v>0.36438593036254635</v>
       </c>
-      <c r="R54" s="220"/>
+      <c r="R54" s="215"/>
     </row>
     <row r="55" spans="6:18" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="K55" s="157" t="s">
@@ -41951,7 +44649,7 @@
         <f t="shared" si="70"/>
         <v>5.9360049763360024E+16</v>
       </c>
-      <c r="R55" s="220"/>
+      <c r="R55" s="215"/>
     </row>
     <row r="56" spans="6:18" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="K56" s="157" t="s">
@@ -41981,7 +44679,7 @@
         <f t="shared" ref="Q56:Q59" si="76">MAX(L56:N56)</f>
         <v>695.4670762888378</v>
       </c>
-      <c r="R56" s="220">
+      <c r="R56" s="215">
         <v>4</v>
       </c>
     </row>
@@ -42013,7 +44711,7 @@
         <f t="shared" si="76"/>
         <v>9337.6615748486856</v>
       </c>
-      <c r="R57" s="220"/>
+      <c r="R57" s="215"/>
     </row>
     <row r="58" spans="6:18" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="K58" s="157" t="s">
@@ -42043,7 +44741,7 @@
         <f t="shared" si="76"/>
         <v>725.36551092066441</v>
       </c>
-      <c r="R58" s="220"/>
+      <c r="R58" s="215"/>
     </row>
     <row r="59" spans="6:18" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="K59" s="157" t="s">
@@ -42073,7 +44771,7 @@
         <f t="shared" si="76"/>
         <v>5.5428405575643274E+20</v>
       </c>
-      <c r="R59" s="220"/>
+      <c r="R59" s="215"/>
     </row>
     <row r="60" spans="6:18" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="K60" s="157" t="s">
@@ -42103,7 +44801,7 @@
         <f t="shared" ref="Q60:Q67" si="80">MAX(L60:N60)</f>
         <v>0.9587815602179951</v>
       </c>
-      <c r="R60" s="220">
+      <c r="R60" s="215">
         <v>2</v>
       </c>
     </row>
@@ -42135,7 +44833,7 @@
         <f t="shared" si="80"/>
         <v>12.873043223404617</v>
       </c>
-      <c r="R61" s="220"/>
+      <c r="R61" s="215"/>
     </row>
     <row r="62" spans="6:18" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="K62" s="157" t="s">
@@ -42165,7 +44863,7 @@
         <f t="shared" si="80"/>
         <v>0.12338257583190283</v>
       </c>
-      <c r="R62" s="220"/>
+      <c r="R62" s="215"/>
     </row>
     <row r="63" spans="6:18" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="K63" s="157" t="s">
@@ -42195,7 +44893,7 @@
         <f t="shared" si="80"/>
         <v>7.6414448634718246E+17</v>
       </c>
-      <c r="R63" s="220"/>
+      <c r="R63" s="215"/>
     </row>
     <row r="64" spans="6:18" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="K64" s="157" t="s">
@@ -42225,7 +44923,7 @@
         <f t="shared" si="80"/>
         <v>1.2822153185194888E-5</v>
       </c>
-      <c r="R64" s="220">
+      <c r="R64" s="215">
         <v>0</v>
       </c>
     </row>
@@ -42257,7 +44955,7 @@
         <f t="shared" si="80"/>
         <v>1.5456205695224421E-4</v>
       </c>
-      <c r="R65" s="220"/>
+      <c r="R65" s="215"/>
     </row>
     <row r="66" spans="11:18" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="K66" s="157" t="s">
@@ -42287,7 +44985,7 @@
         <f t="shared" si="80"/>
         <v>1.7715723362402585E-6</v>
       </c>
-      <c r="R66" s="220"/>
+      <c r="R66" s="215"/>
     </row>
     <row r="67" spans="11:18" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="K67" s="157" t="s">
@@ -42317,7 +45015,7 @@
         <f t="shared" si="80"/>
         <v>1.5311630827938866E-5</v>
       </c>
-      <c r="R67" s="220"/>
+      <c r="R67" s="215"/>
     </row>
     <row r="68" spans="11:18" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="L68" s="6"/>
@@ -42329,11 +45027,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="R48:R51"/>
-    <mergeCell ref="R52:R55"/>
-    <mergeCell ref="R56:R59"/>
-    <mergeCell ref="R60:R63"/>
-    <mergeCell ref="R64:R67"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="F2:J2"/>
     <mergeCell ref="K46:R46"/>
@@ -42345,6 +45038,11 @@
     <mergeCell ref="U28:U33"/>
     <mergeCell ref="U34:U39"/>
     <mergeCell ref="U40:U45"/>
+    <mergeCell ref="R48:R51"/>
+    <mergeCell ref="R52:R55"/>
+    <mergeCell ref="R56:R59"/>
+    <mergeCell ref="R60:R63"/>
+    <mergeCell ref="R64:R67"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>